<commit_message>
257 sheet: BN39-02706A confirmed from user-supplied search results
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GqspcdoB39p9nTcqgMudzj
</commit_message>
<xml_diff>
--- a/Samsung_257_H1_titles.xlsx
+++ b/Samsung_257_H1_titles.xlsx
@@ -473,29 +473,29 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>Samsung</t>
-        </is>
-      </c>
-      <c r="B2" s="2" t="inlineStr">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Samsung</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
         <is>
           <t>BN39-02706A</t>
         </is>
       </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>Samsung TV Cable - BN39-02706A</t>
-        </is>
-      </c>
-      <c r="D2" s="2" t="inlineStr">
-        <is>
-          <t>Low (inferred from series)</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>INFERRED: part type taken from the part-number series; this exact part was not found in any listing. Verify before publishing.</t>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Samsung TV Power Lead Connector - BN39-02706A</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Confirmed from search results you supplied: samsungparts.com, samsungpartsusa.com, iFixit, Impact Computers, FixPart all list it as "Lead Connector Power" (Samsung QN900A/QN800A/QN95A TVs)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
257 sheet: merge extended-search results (92 parts newly identified by exact part number)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GqspcdoB39p9nTcqgMudzj
</commit_message>
<xml_diff>
--- a/Samsung_257_H1_titles.xlsx
+++ b/Samsung_257_H1_titles.xlsx
@@ -500,29 +500,29 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>Samsung</t>
-        </is>
-      </c>
-      <c r="B3" s="2" t="inlineStr">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>Samsung</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
         <is>
           <t>BN39-02310B</t>
         </is>
       </c>
-      <c r="C3" s="2" t="inlineStr">
-        <is>
-          <t>Samsung TV Cable - BN39-02310B</t>
-        </is>
-      </c>
-      <c r="D3" s="2" t="inlineStr">
-        <is>
-          <t>Low (inferred from series)</t>
-        </is>
-      </c>
-      <c r="E3" s="2" t="inlineStr">
-        <is>
-          <t>INFERRED: part type taken from the part-number series; this exact part was not found in any listing. Verify before publishing.</t>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>Samsung TV Dimming Lead Connector - BN39-02310B</t>
+        </is>
+      </c>
+      <c r="D3" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E3" s="4" t="inlineStr">
+        <is>
+          <t>Exact PN found via extended search: "Lead Connector (dimming)" (fits Samsung QN75Q8CAMFXZA-AA01) [searspartsdirect.com] - single/summary-level source; verify.</t>
         </is>
       </c>
     </row>
@@ -554,56 +554,56 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="inlineStr">
-        <is>
-          <t>Samsung</t>
-        </is>
-      </c>
-      <c r="B5" s="2" t="inlineStr">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Samsung</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
         <is>
           <t>BN39-02583A</t>
         </is>
       </c>
-      <c r="C5" s="2" t="inlineStr">
-        <is>
-          <t>Samsung TV Cable - BN39-02583A</t>
-        </is>
-      </c>
-      <c r="D5" s="2" t="inlineStr">
-        <is>
-          <t>Low (inferred from series)</t>
-        </is>
-      </c>
-      <c r="E5" s="2" t="inlineStr">
-        <is>
-          <t>INFERRED: part type taken from the part-number series; this exact part was not found in any listing. Verify before publishing.</t>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Samsung TV One Connect Power Connector Lead - BN39-02583A</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Exact PN found via extended search: "TV One Connect Power Connector Lead" [statewideapp.com.au]</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="2" t="inlineStr">
-        <is>
-          <t>Samsung</t>
-        </is>
-      </c>
-      <c r="B6" s="2" t="inlineStr">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>Samsung</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
         <is>
           <t>BA96-08730A</t>
         </is>
       </c>
-      <c r="C6" s="2" t="inlineStr">
-        <is>
-          <t>Samsung Laptop LCD Assembly - BA96-08730A</t>
-        </is>
-      </c>
-      <c r="D6" s="2" t="inlineStr">
-        <is>
-          <t>Low (inferred from series)</t>
-        </is>
-      </c>
-      <c r="E6" s="2" t="inlineStr">
-        <is>
-          <t>INFERRED: part type taken from the part-number series; this exact part was not found in any listing. Verify before publishing.</t>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>Samsung Laptop Battery Assembly - BA96-08730A</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E6" s="4" t="inlineStr">
+        <is>
+          <t>Exact PN found via extended search: "assy battery-GB5 15_SVC (laptop battery)" (fits GB5-15) [fixpart.co.uk] - single/summary-level source; verify.</t>
         </is>
       </c>
     </row>
@@ -635,29 +635,29 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="2" t="inlineStr">
-        <is>
-          <t>Samsung</t>
-        </is>
-      </c>
-      <c r="B8" s="2" t="inlineStr">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Samsung</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
         <is>
           <t>BN39-02930A</t>
         </is>
       </c>
-      <c r="C8" s="2" t="inlineStr">
-        <is>
-          <t>Samsung TV Cable - BN39-02930A</t>
-        </is>
-      </c>
-      <c r="D8" s="2" t="inlineStr">
-        <is>
-          <t>Low (inferred from series)</t>
-        </is>
-      </c>
-      <c r="E8" s="2" t="inlineStr">
-        <is>
-          <t>INFERRED: part type taken from the part-number series; this exact part was not found in any listing. Verify before publishing.</t>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Samsung TV Power Lead Connector - BN39-02930A</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Exact PN found via extended search: "TV Power Lead Connector" (fits Samsung 49-inch LS49CG934SEXXY, LS49CG954SEXXY, LS49DG910SEXXY, LS49DG930SEXXY, S49CG934SE, S49CG954SE, S49DG910SE, S49DG930SE) [samsungparts.nz]</t>
         </is>
       </c>
     </row>
@@ -689,29 +689,29 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="2" t="inlineStr">
-        <is>
-          <t>Samsung</t>
-        </is>
-      </c>
-      <c r="B10" s="2" t="inlineStr">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>Samsung</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="inlineStr">
         <is>
           <t>BN39-02546A</t>
         </is>
       </c>
-      <c r="C10" s="2" t="inlineStr">
-        <is>
-          <t>Samsung TV Cable - BN39-02546A</t>
-        </is>
-      </c>
-      <c r="D10" s="2" t="inlineStr">
-        <is>
-          <t>Low (inferred from series)</t>
-        </is>
-      </c>
-      <c r="E10" s="2" t="inlineStr">
-        <is>
-          <t>INFERRED: part type taken from the part-number series; this exact part was not found in any listing. Verify before publishing.</t>
+      <c r="C10" s="4" t="inlineStr">
+        <is>
+          <t>Samsung TV LED Bar Connector Cable - BN39-02546A</t>
+        </is>
+      </c>
+      <c r="D10" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E10" s="4" t="inlineStr">
+        <is>
+          <t>Exact PN found via extended search: "Cabo Conector das Barras de Led (LED bar connector cable)" (fits Samsung UN70AU7700G, UN70CU7700G) [lojadotecnico.com] - single/summary-level source; verify.</t>
         </is>
       </c>
     </row>
@@ -743,29 +743,29 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="2" t="inlineStr">
-        <is>
-          <t>Samsung</t>
-        </is>
-      </c>
-      <c r="B12" s="2" t="inlineStr">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Samsung</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
         <is>
           <t>BN39-02465B</t>
         </is>
       </c>
-      <c r="C12" s="2" t="inlineStr">
-        <is>
-          <t>Samsung TV Cable - BN39-02465B</t>
-        </is>
-      </c>
-      <c r="D12" s="2" t="inlineStr">
-        <is>
-          <t>Low (inferred from series)</t>
-        </is>
-      </c>
-      <c r="E12" s="2" t="inlineStr">
-        <is>
-          <t>INFERRED: part type taken from the part-number series; this exact part was not found in any listing. Verify before publishing.</t>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Samsung TV Sub Assembly Lead Connector - BN39-02465B</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Exact PN found via extended search: "Lead Connector-Sub Assembly" (fits Samsung 65/75/82 Q70) [spares2repair.co.uk]</t>
         </is>
       </c>
     </row>
@@ -843,29 +843,29 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="2" t="inlineStr">
-        <is>
-          <t>Samsung</t>
-        </is>
-      </c>
-      <c r="B16" s="2" t="inlineStr">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Samsung</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
         <is>
           <t>BN39-02465A</t>
         </is>
       </c>
-      <c r="C16" s="2" t="inlineStr">
-        <is>
-          <t>Samsung TV Cable - BN39-02465A</t>
-        </is>
-      </c>
-      <c r="D16" s="2" t="inlineStr">
-        <is>
-          <t>Low (inferred from series)</t>
-        </is>
-      </c>
-      <c r="E16" s="2" t="inlineStr">
-        <is>
-          <t>INFERRED: part type taken from the part-number series; this exact part was not found in any listing. Verify before publishing.</t>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Samsung TV Sub Lead Connector - BN39-02465A</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Exact PN found via extended search: "TV Sub Lead Connector" [appliancespares.nz]</t>
         </is>
       </c>
     </row>
@@ -893,56 +893,56 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="2" t="inlineStr">
-        <is>
-          <t>Samsung</t>
-        </is>
-      </c>
-      <c r="B18" s="2" t="inlineStr">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>Samsung</t>
+        </is>
+      </c>
+      <c r="B18" s="4" t="inlineStr">
         <is>
           <t>BN39-01473D</t>
         </is>
       </c>
-      <c r="C18" s="2" t="inlineStr">
-        <is>
-          <t>Samsung TV Cable - BN39-01473D</t>
-        </is>
-      </c>
-      <c r="D18" s="2" t="inlineStr">
-        <is>
-          <t>Low (inferred from series)</t>
-        </is>
-      </c>
-      <c r="E18" s="2" t="inlineStr">
-        <is>
-          <t>INFERRED: part type taken from the part-number series; this exact part was not found in any listing. Verify before publishing.</t>
+      <c r="C18" s="4" t="inlineStr">
+        <is>
+          <t>Samsung TV Flat Lead Connector - BN39-01473D</t>
+        </is>
+      </c>
+      <c r="D18" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E18" s="4" t="inlineStr">
+        <is>
+          <t>Exact PN found via extended search: "LEAD CONNECTOR;UN55C6000,FLAT CONNECTOR" (fits UN55C6000) [samsungpartsusa.com / reliableparts.ca] - single/summary-level source; verify.</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="2" t="inlineStr">
-        <is>
-          <t>Samsung</t>
-        </is>
-      </c>
-      <c r="B19" s="2" t="inlineStr">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Samsung</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
         <is>
           <t>BN39-02469A</t>
         </is>
       </c>
-      <c r="C19" s="2" t="inlineStr">
-        <is>
-          <t>Samsung TV Cable - BN39-02469A</t>
-        </is>
-      </c>
-      <c r="D19" s="2" t="inlineStr">
-        <is>
-          <t>Low (inferred from series)</t>
-        </is>
-      </c>
-      <c r="E19" s="2" t="inlineStr">
-        <is>
-          <t>INFERRED: part type taken from the part-number series; this exact part was not found in any listing. Verify before publishing.</t>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Samsung TV Sub Assembly Lead Connector - BN39-02469A</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>Exact PN found via extended search: "Lead Connector Sub Assy" [shop.digicare.co.uk]</t>
         </is>
       </c>
     </row>
@@ -1009,7 +1009,7 @@
       </c>
       <c r="C22" s="4" t="inlineStr">
         <is>
-          <t>Samsung AC Power Cord - BN39-00141A</t>
+          <t>Samsung Power Cord - BN39-00141A</t>
         </is>
       </c>
       <c r="D22" s="4" t="inlineStr">
@@ -1019,7 +1019,7 @@
       </c>
       <c r="E22" s="4" t="inlineStr">
         <is>
-          <t>samsungparts.com page; part type from listing summary</t>
+          <t>Exact PN found via extended search: "Power Cord" [impactcomputers.com] - single/summary-level source; verify.</t>
         </is>
       </c>
     </row>
@@ -1051,29 +1051,29 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="2" t="inlineStr">
-        <is>
-          <t>Samsung</t>
-        </is>
-      </c>
-      <c r="B24" s="2" t="inlineStr">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Samsung</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
         <is>
           <t>AH91-09169Z</t>
         </is>
       </c>
-      <c r="C24" s="2" t="inlineStr">
-        <is>
-          <t>Samsung Soundbar Speaker Assembly - AH91-09169Z</t>
-        </is>
-      </c>
-      <c r="D24" s="2" t="inlineStr">
-        <is>
-          <t>Low (inferred from series)</t>
-        </is>
-      </c>
-      <c r="E24" s="2" t="inlineStr">
-        <is>
-          <t>INFERRED: part type taken from the part-number series; this exact part was not found in any listing. Verify before publishing.</t>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Samsung Speaker Subwoofer - AH91-09169Z</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>Exact PN found via extended search: "Speaker Subwoofer" (fits Samsung HW-Q800C/ZA soundbar) [impactcomputers.com]</t>
         </is>
       </c>
     </row>
@@ -1090,44 +1090,44 @@
       </c>
       <c r="C25" s="4" t="inlineStr">
         <is>
-          <t>Samsung TV Lead Connector Sub Assembly - BN39-02231A</t>
+          <t>Samsung TV Sub Assembly Lead Connector - BN39-02231A</t>
         </is>
       </c>
       <c r="D25" s="4" t="inlineStr">
         <is>
-          <t>Medium (revision of confirmed part)</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="E25" s="4" t="inlineStr">
         <is>
-          <t>Same base number as confirmed BN39-02231D (different suffix letter = revision); type taken from that part. Exact-number listing not found.</t>
+          <t>Exact PN found via extended search: "Lead Connector-Sub Assembly" (fits Samsung QN75Q6FNAFXZA) [shopjimmy.com] - single/summary-level source; verify.</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="2" t="inlineStr">
-        <is>
-          <t>Samsung</t>
-        </is>
-      </c>
-      <c r="B26" s="2" t="inlineStr">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Samsung</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
         <is>
           <t>BN39-01744H</t>
         </is>
       </c>
-      <c r="C26" s="2" t="inlineStr">
-        <is>
-          <t>Samsung TV Cable - BN39-01744H</t>
-        </is>
-      </c>
-      <c r="D26" s="2" t="inlineStr">
-        <is>
-          <t>Low (inferred from series)</t>
-        </is>
-      </c>
-      <c r="E26" s="2" t="inlineStr">
-        <is>
-          <t>INFERRED: part type taken from the part-number series; this exact part was not found in any listing. Verify before publishing.</t>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Samsung TV Lead Connector - BN39-01744H</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>Exact PN found via extended search: "Lead Connector (40 46 FHD)" (fits Samsung UE46F5500AW; UN46F6300AF/XZA (PartStore)) [sparessamsung.com]</t>
         </is>
       </c>
     </row>
@@ -1455,29 +1455,29 @@
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="2" t="inlineStr">
-        <is>
-          <t>Samsung</t>
-        </is>
-      </c>
-      <c r="B40" s="2" t="inlineStr">
+      <c r="A40" s="4" t="inlineStr">
+        <is>
+          <t>Samsung</t>
+        </is>
+      </c>
+      <c r="B40" s="4" t="inlineStr">
         <is>
           <t>BN39-00185A</t>
         </is>
       </c>
-      <c r="C40" s="2" t="inlineStr">
-        <is>
-          <t>Samsung TV Cable - BN39-00185A</t>
-        </is>
-      </c>
-      <c r="D40" s="2" t="inlineStr">
-        <is>
-          <t>Low (inferred from series)</t>
-        </is>
-      </c>
-      <c r="E40" s="2" t="inlineStr">
-        <is>
-          <t>INFERRED: part type taken from the part-number series; this exact part was not found in any listing. Verify before publishing.</t>
+      <c r="C40" s="4" t="inlineStr">
+        <is>
+          <t>Samsung TV Power Cord - BN39-00185A</t>
+        </is>
+      </c>
+      <c r="D40" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E40" s="4" t="inlineStr">
+        <is>
+          <t>Exact PN found via extended search: "POWER CORD-DT" [unlimitedapplianceparts.com] - single/summary-level source; verify.</t>
         </is>
       </c>
     </row>
@@ -1578,29 +1578,29 @@
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="2" t="inlineStr">
-        <is>
-          <t>Samsung</t>
-        </is>
-      </c>
-      <c r="B45" s="2" t="inlineStr">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>Samsung</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
         <is>
           <t>BN39-02752A</t>
         </is>
       </c>
-      <c r="C45" s="2" t="inlineStr">
-        <is>
-          <t>Samsung TV Cable - BN39-02752A</t>
-        </is>
-      </c>
-      <c r="D45" s="2" t="inlineStr">
-        <is>
-          <t>Low (inferred from series)</t>
-        </is>
-      </c>
-      <c r="E45" s="2" t="inlineStr">
-        <is>
-          <t>INFERRED: part type taken from the part-number series; this exact part was not found in any listing. Verify before publishing.</t>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>Samsung TV AC Power Cable - BN39-02752A</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>Exact PN found via extended search: "AC Power Cable" (fits Samsung TV) [shop.digicare.co.uk]</t>
         </is>
       </c>
     </row>
@@ -1794,17 +1794,17 @@
       </c>
       <c r="C53" s="4" t="inlineStr">
         <is>
-          <t>Samsung TV Sub Lead Connector Assembly - BN39-02457A</t>
+          <t>Samsung TV Main Board to IR Receiver and Power Switch Cable - BN39-02457A</t>
         </is>
       </c>
       <c r="D53" s="4" t="inlineStr">
         <is>
-          <t>Medium (revision of confirmed part)</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="E53" s="4" t="inlineStr">
         <is>
-          <t>Same base number as confirmed BN39-02457B (different suffix letter = revision); type taken from that part. Exact-number listing not found.</t>
+          <t>Exact PN found via extended search: "Przewod (cable) connecting main board to IR receiver and power switch" (fits Samsung UE43RU7102KXXH) [mimelectronics.pl] - single/summary-level source; verify.</t>
         </is>
       </c>
     </row>
@@ -1936,29 +1936,29 @@
       </c>
     </row>
     <row r="59">
-      <c r="A59" s="2" t="inlineStr">
-        <is>
-          <t>Samsung</t>
-        </is>
-      </c>
-      <c r="B59" s="2" t="inlineStr">
+      <c r="A59" s="4" t="inlineStr">
+        <is>
+          <t>Samsung</t>
+        </is>
+      </c>
+      <c r="B59" s="4" t="inlineStr">
         <is>
           <t>BN39-02618A</t>
         </is>
       </c>
-      <c r="C59" s="2" t="inlineStr">
-        <is>
-          <t>Samsung TV Cable - BN39-02618A</t>
-        </is>
-      </c>
-      <c r="D59" s="2" t="inlineStr">
-        <is>
-          <t>Low (inferred from series)</t>
-        </is>
-      </c>
-      <c r="E59" s="2" t="inlineStr">
-        <is>
-          <t>INFERRED: part type taken from the part-number series; this exact part was not found in any listing. Verify before publishing.</t>
+      <c r="C59" s="4" t="inlineStr">
+        <is>
+          <t>Samsung TV Lead Connector - BN39-02618A</t>
+        </is>
+      </c>
+      <c r="D59" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E59" s="4" t="inlineStr">
+        <is>
+          <t>Exact PN found via extended search: "Lead Connector-Etc;Ul210166P" [samsungpartsusa.com] - single/summary-level source; verify.</t>
         </is>
       </c>
     </row>
@@ -1975,7 +1975,7 @@
       </c>
       <c r="C60" s="4" t="inlineStr">
         <is>
-          <t>Samsung TV Power Cable Connector - BN39-01884H</t>
+          <t>Samsung TV Power Lead Connector - BN39-01884H</t>
         </is>
       </c>
       <c r="D60" s="4" t="inlineStr">
@@ -1985,7 +1985,7 @@
       </c>
       <c r="E60" s="4" t="inlineStr">
         <is>
-          <t>samsungpartsusa.com page; part type from listing summary</t>
+          <t>Exact PN found via extended search: "Lead Connector-Power" [ebay.com] - single/summary-level source; verify.</t>
         </is>
       </c>
     </row>
@@ -2013,56 +2013,56 @@
       </c>
     </row>
     <row r="62">
-      <c r="A62" s="2" t="inlineStr">
-        <is>
-          <t>Samsung</t>
-        </is>
-      </c>
-      <c r="B62" s="2" t="inlineStr">
+      <c r="A62" s="4" t="inlineStr">
+        <is>
+          <t>Samsung</t>
+        </is>
+      </c>
+      <c r="B62" s="4" t="inlineStr">
         <is>
           <t>BN39-02821A</t>
         </is>
       </c>
-      <c r="C62" s="2" t="inlineStr">
-        <is>
-          <t>Samsung TV Cable - BN39-02821A</t>
-        </is>
-      </c>
-      <c r="D62" s="2" t="inlineStr">
-        <is>
-          <t>Low (inferred from series)</t>
-        </is>
-      </c>
-      <c r="E62" s="2" t="inlineStr">
-        <is>
-          <t>INFERRED: part type taken from the part-number series; this exact part was not found in any listing. Verify before publishing.</t>
+      <c r="C62" s="4" t="inlineStr">
+        <is>
+          <t>Samsung TV Power Lead Connector - BN39-02821A</t>
+        </is>
+      </c>
+      <c r="D62" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E62" s="4" t="inlineStr">
+        <is>
+          <t>Exact PN found via extended search: "LEAD CONNECTOR-POWER" (fits QN65QN800BFXZA) [ued.net] - single/summary-level source; verify.</t>
         </is>
       </c>
     </row>
     <row r="63">
-      <c r="A63" s="2" t="inlineStr">
-        <is>
-          <t>Samsung</t>
-        </is>
-      </c>
-      <c r="B63" s="2" t="inlineStr">
+      <c r="A63" s="4" t="inlineStr">
+        <is>
+          <t>Samsung</t>
+        </is>
+      </c>
+      <c r="B63" s="4" t="inlineStr">
         <is>
           <t>BN39-02692A</t>
         </is>
       </c>
-      <c r="C63" s="2" t="inlineStr">
-        <is>
-          <t>Samsung TV Cable - BN39-02692A</t>
-        </is>
-      </c>
-      <c r="D63" s="2" t="inlineStr">
-        <is>
-          <t>Low (inferred from series)</t>
-        </is>
-      </c>
-      <c r="E63" s="2" t="inlineStr">
-        <is>
-          <t>INFERRED: part type taken from the part-number series; this exact part was not found in any listing. Verify before publishing.</t>
+      <c r="C63" s="4" t="inlineStr">
+        <is>
+          <t>Samsung TV Sub Assembly Lead Connector - BN39-02692A</t>
+        </is>
+      </c>
+      <c r="D63" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E63" s="4" t="inlineStr">
+        <is>
+          <t>Exact PN found via extended search: "LEAD CONNECTOR-SUB ASSY;LS03A,UL21451,10" [ued.net] - single/summary-level source; verify.</t>
         </is>
       </c>
     </row>
@@ -2084,12 +2084,12 @@
       </c>
       <c r="D64" s="4" t="inlineStr">
         <is>
-          <t>Medium (revision of confirmed part)</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="E64" s="4" t="inlineStr">
         <is>
-          <t>Same base number as confirmed BN39-02207C (different suffix letter = revision); type taken from that part. Exact-number listing not found.</t>
+          <t>Exact PN found via extended search: "Cabo Conexao da Principal x Placa Fonte (Lead Connector-Power)" (fits QN55Q90TD) [comclick.com.br] - single/summary-level source; verify.</t>
         </is>
       </c>
     </row>
@@ -2194,52 +2194,56 @@
       </c>
     </row>
     <row r="69">
-      <c r="A69" s="3" t="inlineStr">
-        <is>
-          <t>Samsung</t>
-        </is>
-      </c>
-      <c r="B69" s="3" t="inlineStr">
+      <c r="A69" s="4" t="inlineStr">
+        <is>
+          <t>Samsung</t>
+        </is>
+      </c>
+      <c r="B69" s="4" t="inlineStr">
         <is>
           <t>AH81-15587A</t>
         </is>
       </c>
-      <c r="C69" s="3" t="n"/>
-      <c r="D69" s="3" t="inlineStr">
-        <is>
-          <t>Needs review</t>
-        </is>
-      </c>
-      <c r="E69" s="3" t="inlineStr">
-        <is>
-          <t>No listing and no reliable series pattern; not guessed.</t>
+      <c r="C69" s="4" t="inlineStr">
+        <is>
+          <t>Samsung Service Power Cord - AH81-15587A</t>
+        </is>
+      </c>
+      <c r="D69" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E69" s="4" t="inlineStr">
+        <is>
+          <t>Exact PN found via extended search: "Service JDM power cord" [samsungparts.com] - single/summary-level source; verify.</t>
         </is>
       </c>
     </row>
     <row r="70">
-      <c r="A70" s="2" t="inlineStr">
-        <is>
-          <t>Samsung</t>
-        </is>
-      </c>
-      <c r="B70" s="2" t="inlineStr">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>Samsung</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
         <is>
           <t>BN39-02312A</t>
         </is>
       </c>
-      <c r="C70" s="2" t="inlineStr">
-        <is>
-          <t>Samsung TV Cable - BN39-02312A</t>
-        </is>
-      </c>
-      <c r="D70" s="2" t="inlineStr">
-        <is>
-          <t>Low (inferred from series)</t>
-        </is>
-      </c>
-      <c r="E70" s="2" t="inlineStr">
-        <is>
-          <t>INFERRED: part type taken from the part-number series; this exact part was not found in any listing. Verify before publishing.</t>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>Samsung TV One Connect Sub Assembly Lead Connector - BN39-02312A</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>Exact PN found via extended search: "One Connect cable (Lead Connector-Sub Assembly)" (fits Samsung Q7C/Q7F QLED (e.g. QE65Q7FAMTXXH)) [allegro.pl]</t>
         </is>
       </c>
     </row>
@@ -2317,29 +2321,29 @@
       </c>
     </row>
     <row r="74">
-      <c r="A74" s="2" t="inlineStr">
-        <is>
-          <t>Samsung</t>
-        </is>
-      </c>
-      <c r="B74" s="2" t="inlineStr">
+      <c r="A74" s="4" t="inlineStr">
+        <is>
+          <t>Samsung</t>
+        </is>
+      </c>
+      <c r="B74" s="4" t="inlineStr">
         <is>
           <t>AH91-00842A</t>
         </is>
       </c>
-      <c r="C74" s="2" t="inlineStr">
-        <is>
-          <t>Samsung Soundbar Speaker Assembly - AH91-00842A</t>
-        </is>
-      </c>
-      <c r="D74" s="2" t="inlineStr">
-        <is>
-          <t>Low (inferred from series)</t>
-        </is>
-      </c>
-      <c r="E74" s="2" t="inlineStr">
-        <is>
-          <t>INFERRED: part type taken from the part-number series; this exact part was not found in any listing. Verify before publishing.</t>
+      <c r="C74" s="4" t="inlineStr">
+        <is>
+          <t>Samsung Soundbar Subwoofer Speaker Assembly - AH91-00842A</t>
+        </is>
+      </c>
+      <c r="D74" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E74" s="4" t="inlineStr">
+        <is>
+          <t>Exact PN found via extended search: "Assy Speaker-Subwoofer" (fits HW-J550) [tvserviceparts.com] - single/summary-level source; verify.</t>
         </is>
       </c>
     </row>
@@ -2394,29 +2398,29 @@
       </c>
     </row>
     <row r="77">
-      <c r="A77" s="2" t="inlineStr">
-        <is>
-          <t>Samsung</t>
-        </is>
-      </c>
-      <c r="B77" s="2" t="inlineStr">
+      <c r="A77" s="4" t="inlineStr">
+        <is>
+          <t>Samsung</t>
+        </is>
+      </c>
+      <c r="B77" s="4" t="inlineStr">
         <is>
           <t>BN39-02669A</t>
         </is>
       </c>
-      <c r="C77" s="2" t="inlineStr">
-        <is>
-          <t>Samsung TV Cable - BN39-02669A</t>
-        </is>
-      </c>
-      <c r="D77" s="2" t="inlineStr">
-        <is>
-          <t>Low (inferred from series)</t>
-        </is>
-      </c>
-      <c r="E77" s="2" t="inlineStr">
-        <is>
-          <t>INFERRED: part type taken from the part-number series; this exact part was not found in any listing. Verify before publishing.</t>
+      <c r="C77" s="4" t="inlineStr">
+        <is>
+          <t>Samsung TV Backlight Lead Connector - BN39-02669A</t>
+        </is>
+      </c>
+      <c r="D77" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E77" s="4" t="inlineStr">
+        <is>
+          <t>Exact PN found via extended search: "LEAD CONNECTOR-BLU;UL21016" (fits 65AU8500/8000) [ued.net] - single/summary-level source; verify.</t>
         </is>
       </c>
     </row>
@@ -2525,29 +2529,29 @@
       </c>
     </row>
     <row r="82">
-      <c r="A82" s="2" t="inlineStr">
-        <is>
-          <t>Samsung</t>
-        </is>
-      </c>
-      <c r="B82" s="2" t="inlineStr">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>Samsung</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
         <is>
           <t>BN39-02030C</t>
         </is>
       </c>
-      <c r="C82" s="2" t="inlineStr">
-        <is>
-          <t>Samsung TV Cable - BN39-02030C</t>
-        </is>
-      </c>
-      <c r="D82" s="2" t="inlineStr">
-        <is>
-          <t>Low (inferred from series)</t>
-        </is>
-      </c>
-      <c r="E82" s="2" t="inlineStr">
-        <is>
-          <t>INFERRED: part type taken from the part-number series; this exact part was not found in any listing. Verify before publishing.</t>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>Samsung TV Backlight Lead Connector - BN39-02030C</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>Exact PN found via extended search: "Lead Connector BLU (BLU, UL21016, 16P, 150MM)" (fits Samsung UN55JU / UN55KU series LED TVs (per homedepot.ca lookups)) [impactcomputers.com]</t>
         </is>
       </c>
     </row>
@@ -2575,56 +2579,56 @@
       </c>
     </row>
     <row r="84">
-      <c r="A84" s="2" t="inlineStr">
-        <is>
-          <t>Samsung</t>
-        </is>
-      </c>
-      <c r="B84" s="2" t="inlineStr">
+      <c r="A84" s="4" t="inlineStr">
+        <is>
+          <t>Samsung</t>
+        </is>
+      </c>
+      <c r="B84" s="4" t="inlineStr">
         <is>
           <t>BA98-03492A</t>
         </is>
       </c>
-      <c r="C84" s="2" t="inlineStr">
-        <is>
-          <t>Samsung Laptop Case Assembly - BA98-03492A</t>
-        </is>
-      </c>
-      <c r="D84" s="2" t="inlineStr">
-        <is>
-          <t>Low (inferred from series)</t>
-        </is>
-      </c>
-      <c r="E84" s="2" t="inlineStr">
-        <is>
-          <t>INFERRED: part type taken from the part-number series; this exact part was not found in any listing. Verify before publishing.</t>
+      <c r="C84" s="4" t="inlineStr">
+        <is>
+          <t>Samsung Laptop Rear Protective Cover - BA98-03492A</t>
+        </is>
+      </c>
+      <c r="D84" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E84" s="4" t="inlineStr">
+        <is>
+          <t>Exact PN found via extended search: "rear protective cover for laptop motherboard (VỎ SAU BẢO VỆ BẢN MẠCH MÁY TÍNH XÁCH TAY)" [importgenius.com] - single/summary-level source; verify.</t>
         </is>
       </c>
     </row>
     <row r="85">
-      <c r="A85" s="2" t="inlineStr">
-        <is>
-          <t>Samsung</t>
-        </is>
-      </c>
-      <c r="B85" s="2" t="inlineStr">
+      <c r="A85" s="4" t="inlineStr">
+        <is>
+          <t>Samsung</t>
+        </is>
+      </c>
+      <c r="B85" s="4" t="inlineStr">
         <is>
           <t>BN39-02563D</t>
         </is>
       </c>
-      <c r="C85" s="2" t="inlineStr">
-        <is>
-          <t>Samsung TV Cable - BN39-02563D</t>
-        </is>
-      </c>
-      <c r="D85" s="2" t="inlineStr">
-        <is>
-          <t>Low (inferred from series)</t>
-        </is>
-      </c>
-      <c r="E85" s="2" t="inlineStr">
-        <is>
-          <t>INFERRED: part type taken from the part-number series; this exact part was not found in any listing. Verify before publishing.</t>
+      <c r="C85" s="4" t="inlineStr">
+        <is>
+          <t>Samsung TV Sub Assembly Lead Connector - BN39-02563D</t>
+        </is>
+      </c>
+      <c r="D85" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E85" s="4" t="inlineStr">
+        <is>
+          <t>Exact PN found via extended search: "Lead Connector-Sub Assy" [shop.app (SilverShopTvParts)] - single/summary-level source; verify.</t>
         </is>
       </c>
     </row>
@@ -2710,29 +2714,29 @@
       </c>
     </row>
     <row r="89">
-      <c r="A89" s="2" t="inlineStr">
-        <is>
-          <t>Samsung</t>
-        </is>
-      </c>
-      <c r="B89" s="2" t="inlineStr">
+      <c r="A89" s="4" t="inlineStr">
+        <is>
+          <t>Samsung</t>
+        </is>
+      </c>
+      <c r="B89" s="4" t="inlineStr">
         <is>
           <t>BA96-08604A</t>
         </is>
       </c>
-      <c r="C89" s="2" t="inlineStr">
-        <is>
-          <t>Samsung Laptop LCD Assembly - BA96-08604A</t>
-        </is>
-      </c>
-      <c r="D89" s="2" t="inlineStr">
-        <is>
-          <t>Low (inferred from series)</t>
-        </is>
-      </c>
-      <c r="E89" s="2" t="inlineStr">
-        <is>
-          <t>INFERRED: part type taken from the part-number series; this exact part was not found in any listing. Verify before publishing.</t>
+      <c r="C89" s="4" t="inlineStr">
+        <is>
+          <t>Samsung Laptop Palmrest Cover with Keyboard - BA96-08604A</t>
+        </is>
+      </c>
+      <c r="D89" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E89" s="4" t="inlineStr">
+        <is>
+          <t>Exact PN found via extended search: "Palmrest cover with UK keyboard" (fits Samsung Galaxy Book4 Pro NP960XGK) [ebay.ca] - single/summary-level source; verify.</t>
         </is>
       </c>
     </row>
@@ -2764,25 +2768,29 @@
       </c>
     </row>
     <row r="91">
-      <c r="A91" s="3" t="inlineStr">
-        <is>
-          <t>Samsung</t>
-        </is>
-      </c>
-      <c r="B91" s="3" t="inlineStr">
+      <c r="A91" s="4" t="inlineStr">
+        <is>
+          <t>Samsung</t>
+        </is>
+      </c>
+      <c r="B91" s="4" t="inlineStr">
         <is>
           <t>AH81-17534A</t>
         </is>
       </c>
-      <c r="C91" s="3" t="n"/>
-      <c r="D91" s="3" t="inlineStr">
-        <is>
-          <t>Needs review</t>
-        </is>
-      </c>
-      <c r="E91" s="3" t="inlineStr">
-        <is>
-          <t>No listing and no reliable series pattern; not guessed.</t>
+      <c r="C91" s="4" t="inlineStr">
+        <is>
+          <t>Samsung Service Power Cord - AH81-17534A</t>
+        </is>
+      </c>
+      <c r="D91" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E91" s="4" t="inlineStr">
+        <is>
+          <t>Exact PN found via extended search: "SVC JDM-POWER CORD" (fits Samsung HW-B550D soundbar/subwoofer (user guide lists it as power cord)) [samsungersatzteile.com] - single/summary-level source; verify.</t>
         </is>
       </c>
     </row>
@@ -2810,29 +2818,29 @@
       </c>
     </row>
     <row r="93">
-      <c r="A93" s="2" t="inlineStr">
-        <is>
-          <t>Samsung</t>
-        </is>
-      </c>
-      <c r="B93" s="2" t="inlineStr">
+      <c r="A93" s="4" t="inlineStr">
+        <is>
+          <t>Samsung</t>
+        </is>
+      </c>
+      <c r="B93" s="4" t="inlineStr">
         <is>
           <t>BA98-03735A</t>
         </is>
       </c>
-      <c r="C93" s="2" t="inlineStr">
-        <is>
-          <t>Samsung Laptop Case Assembly - BA98-03735A</t>
-        </is>
-      </c>
-      <c r="D93" s="2" t="inlineStr">
-        <is>
-          <t>Low (inferred from series)</t>
-        </is>
-      </c>
-      <c r="E93" s="2" t="inlineStr">
-        <is>
-          <t>INFERRED: part type taken from the part-number series; this exact part was not found in any listing. Verify before publishing.</t>
+      <c r="C93" s="4" t="inlineStr">
+        <is>
+          <t>Samsung Laptop Front Right Rubber Foot - BA98-03735A</t>
+        </is>
+      </c>
+      <c r="D93" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E93" s="4" t="inlineStr">
+        <is>
+          <t>Exact PN found via extended search: "RUBBER FOOT FRONT R" (fits VENUS3 16 notebook (NP960XFH-XA3US)) [impactcomputers.com] - single/summary-level source; verify.</t>
         </is>
       </c>
     </row>
@@ -2864,25 +2872,29 @@
       </c>
     </row>
     <row r="95">
-      <c r="A95" s="3" t="inlineStr">
-        <is>
-          <t>Samsung</t>
-        </is>
-      </c>
-      <c r="B95" s="3" t="inlineStr">
+      <c r="A95" s="4" t="inlineStr">
+        <is>
+          <t>Samsung</t>
+        </is>
+      </c>
+      <c r="B95" s="4" t="inlineStr">
         <is>
           <t>AH96-03468A</t>
         </is>
       </c>
-      <c r="C95" s="3" t="n"/>
-      <c r="D95" s="3" t="inlineStr">
-        <is>
-          <t>Needs review</t>
-        </is>
-      </c>
-      <c r="E95" s="3" t="inlineStr">
-        <is>
-          <t>No listing and no reliable series pattern; not guessed.</t>
+      <c r="C95" s="4" t="inlineStr">
+        <is>
+          <t>Samsung Holder P-Mount - AH96-03468A</t>
+        </is>
+      </c>
+      <c r="D95" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E95" s="4" t="inlineStr">
+        <is>
+          <t>Exact PN found via extended search: "Holder P-Mount; W/W, Pc+A" (fits Samsung HW-J7500/ZA, HW-J7501/ZA, HW-J7501/EN soundbars) [tvserviceparts.com] - single/summary-level source; verify.</t>
         </is>
       </c>
     </row>
@@ -2991,56 +3003,56 @@
       </c>
     </row>
     <row r="100">
-      <c r="A100" s="2" t="inlineStr">
-        <is>
-          <t>Samsung</t>
-        </is>
-      </c>
-      <c r="B100" s="2" t="inlineStr">
+      <c r="A100" s="4" t="inlineStr">
+        <is>
+          <t>Samsung</t>
+        </is>
+      </c>
+      <c r="B100" s="4" t="inlineStr">
         <is>
           <t>BN39-02710A</t>
         </is>
       </c>
-      <c r="C100" s="2" t="inlineStr">
-        <is>
-          <t>Samsung TV Cable - BN39-02710A</t>
-        </is>
-      </c>
-      <c r="D100" s="2" t="inlineStr">
-        <is>
-          <t>Low (inferred from series)</t>
-        </is>
-      </c>
-      <c r="E100" s="2" t="inlineStr">
-        <is>
-          <t>INFERRED: part type taken from the part-number series; this exact part was not found in any listing. Verify before publishing.</t>
+      <c r="C100" s="4" t="inlineStr">
+        <is>
+          <t>Samsung TV Electrical Cable with Connector - BN39-02710A</t>
+        </is>
+      </c>
+      <c r="D100" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E100" s="4" t="inlineStr">
+        <is>
+          <t>Exact PN found via extended search: "electrical cable with connector (about 340mm, below 1000V)" [volza.com] - single/summary-level source; verify.</t>
         </is>
       </c>
     </row>
     <row r="101">
-      <c r="A101" s="2" t="inlineStr">
-        <is>
-          <t>Samsung</t>
-        </is>
-      </c>
-      <c r="B101" s="2" t="inlineStr">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>Samsung</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
         <is>
           <t>BA31-00128A</t>
         </is>
       </c>
-      <c r="C101" s="2" t="inlineStr">
-        <is>
-          <t>Samsung Laptop Fan - BA31-00128A</t>
-        </is>
-      </c>
-      <c r="D101" s="2" t="inlineStr">
-        <is>
-          <t>Low (inferred from series)</t>
-        </is>
-      </c>
-      <c r="E101" s="2" t="inlineStr">
-        <is>
-          <t>INFERRED: part type taken from the part-number series; this exact part was not found in any listing. Verify before publishing.</t>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>Samsung Laptop Right CPU Cooling Fan - BA31-00128A</t>
+        </is>
+      </c>
+      <c r="D101" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t>Exact PN found via extended search: "Right CPU Cooling Fan" (fits Samsung NP700Z7C series laptop) [ebay.com]</t>
         </is>
       </c>
     </row>
@@ -3095,25 +3107,29 @@
       </c>
     </row>
     <row r="104">
-      <c r="A104" s="3" t="inlineStr">
-        <is>
-          <t>Samsung</t>
-        </is>
-      </c>
-      <c r="B104" s="3" t="inlineStr">
+      <c r="A104" s="4" t="inlineStr">
+        <is>
+          <t>Samsung</t>
+        </is>
+      </c>
+      <c r="B104" s="4" t="inlineStr">
         <is>
           <t>3501-001233</t>
         </is>
       </c>
-      <c r="C104" s="3" t="n"/>
-      <c r="D104" s="3" t="inlineStr">
-        <is>
-          <t>Needs review</t>
-        </is>
-      </c>
-      <c r="E104" s="3" t="inlineStr">
-        <is>
-          <t>No listing and no reliable series pattern; not guessed.</t>
+      <c r="C104" s="4" t="inlineStr">
+        <is>
+          <t>Samsung Air Conditioner Miniature Relay - 3501-001233</t>
+        </is>
+      </c>
+      <c r="D104" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E104" s="4" t="inlineStr">
+        <is>
+          <t>Exact PN found via extended search: "miniature relay (220V)" (fits Samsung air conditioner UM18B1C2) [ereplacementparts.com] - single/summary-level source; verify.</t>
         </is>
       </c>
     </row>
@@ -3145,25 +3161,29 @@
       </c>
     </row>
     <row r="106">
-      <c r="A106" s="3" t="inlineStr">
-        <is>
-          <t>Samsung</t>
-        </is>
-      </c>
-      <c r="B106" s="3" t="inlineStr">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>Samsung</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
         <is>
           <t>0505-003755</t>
         </is>
       </c>
-      <c r="C106" s="3" t="n"/>
-      <c r="D106" s="3" t="inlineStr">
-        <is>
-          <t>Needs review</t>
-        </is>
-      </c>
-      <c r="E106" s="3" t="inlineStr">
-        <is>
-          <t>No listing and no reliable series pattern; not guessed.</t>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>Samsung Refrigerator MOSFET - 0505-003755</t>
+        </is>
+      </c>
+      <c r="D106" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E106" t="inlineStr">
+        <is>
+          <t>Exact PN found via extended search: "MOSFET / FET-silicon;aod2910e,n,100v,37a,23mohm" (fits Samsung refrigerators (e.g. RF24BB660012AA), TVs, laptops per catalog lookups) [onderdelenexpert.nl]</t>
         </is>
       </c>
     </row>
@@ -3195,25 +3215,29 @@
       </c>
     </row>
     <row r="108">
-      <c r="A108" s="3" t="inlineStr">
-        <is>
-          <t>Samsung</t>
-        </is>
-      </c>
-      <c r="B108" s="3" t="inlineStr">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>Samsung</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
         <is>
           <t>BN07-01765A</t>
         </is>
       </c>
-      <c r="C108" s="3" t="n"/>
-      <c r="D108" s="3" t="inlineStr">
-        <is>
-          <t>Needs review</t>
-        </is>
-      </c>
-      <c r="E108" s="3" t="inlineStr">
-        <is>
-          <t>No listing and no reliable series pattern; not guessed.</t>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>Samsung TV Screen Panel - BN07-01765A</t>
+        </is>
+      </c>
+      <c r="D108" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E108" t="inlineStr">
+        <is>
+          <t>Exact PN found via extended search: "TV Screen Panel" [appliancespares.nz]</t>
         </is>
       </c>
     </row>
@@ -3291,29 +3315,29 @@
       </c>
     </row>
     <row r="112">
-      <c r="A112" s="2" t="inlineStr">
-        <is>
-          <t>Samsung</t>
-        </is>
-      </c>
-      <c r="B112" s="2" t="inlineStr">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>Samsung</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
         <is>
           <t>BN39-02219A</t>
         </is>
       </c>
-      <c r="C112" s="2" t="inlineStr">
-        <is>
-          <t>Samsung TV Cable - BN39-02219A</t>
-        </is>
-      </c>
-      <c r="D112" s="2" t="inlineStr">
-        <is>
-          <t>Low (inferred from series)</t>
-        </is>
-      </c>
-      <c r="E112" s="2" t="inlineStr">
-        <is>
-          <t>INFERRED: part type taken from the part-number series; this exact part was not found in any listing. Verify before publishing.</t>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>Samsung TV Sub Lead Connector Cable - BN39-02219A</t>
+        </is>
+      </c>
+      <c r="D112" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E112" t="inlineStr">
+        <is>
+          <t>Exact PN found via extended search: "Cable-Lead Connector-Sub (55Ku6500, Ul21016)" (fits Samsung UN55KU6500FXZA, UN55MU6500FXZA and others) [tvserviceparts.com]</t>
         </is>
       </c>
     </row>
@@ -3364,56 +3388,56 @@
       </c>
     </row>
     <row r="115">
-      <c r="A115" s="2" t="inlineStr">
-        <is>
-          <t>Samsung</t>
-        </is>
-      </c>
-      <c r="B115" s="2" t="inlineStr">
+      <c r="A115" s="4" t="inlineStr">
+        <is>
+          <t>Samsung</t>
+        </is>
+      </c>
+      <c r="B115" s="4" t="inlineStr">
         <is>
           <t>BA97-12318A</t>
         </is>
       </c>
-      <c r="C115" s="2" t="inlineStr">
+      <c r="C115" s="4" t="inlineStr">
         <is>
           <t>Samsung Laptop Front Top Case Assembly - BA97-12318A</t>
         </is>
       </c>
-      <c r="D115" s="2" t="inlineStr">
-        <is>
-          <t>Low (inferred from series)</t>
-        </is>
-      </c>
-      <c r="E115" s="2" t="inlineStr">
-        <is>
-          <t>INFERRED: part type taken from the part-number series; this exact part was not found in any listing. Verify before publishing.</t>
+      <c r="D115" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E115" s="4" t="inlineStr">
+        <is>
+          <t>Exact PN found via extended search: "Assembly Case Front-top_svc;mars-13,sec,blue" (fits NP930QDBKE1US) [partstore.encompass.com] - single/summary-level source; verify.</t>
         </is>
       </c>
     </row>
     <row r="116">
-      <c r="A116" s="2" t="inlineStr">
-        <is>
-          <t>Samsung</t>
-        </is>
-      </c>
-      <c r="B116" s="2" t="inlineStr">
+      <c r="A116" s="4" t="inlineStr">
+        <is>
+          <t>Samsung</t>
+        </is>
+      </c>
+      <c r="B116" s="4" t="inlineStr">
         <is>
           <t>BA97-13332A</t>
         </is>
       </c>
-      <c r="C116" s="2" t="inlineStr">
-        <is>
-          <t>Samsung Laptop Front Top Case Assembly - BA97-13332A</t>
-        </is>
-      </c>
-      <c r="D116" s="2" t="inlineStr">
-        <is>
-          <t>Low (inferred from series)</t>
-        </is>
-      </c>
-      <c r="E116" s="2" t="inlineStr">
-        <is>
-          <t>INFERRED: part type taken from the part-number series; this exact part was not found in any listing. Verify before publishing.</t>
+      <c r="C116" s="4" t="inlineStr">
+        <is>
+          <t>Samsung Laptop Front Case Assembly with Touchpad - BA97-13332A</t>
+        </is>
+      </c>
+      <c r="D116" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E116" s="4" t="inlineStr">
+        <is>
+          <t>Exact PN found via extended search: "front case assembly with touchpad (as paraphrased in summary)" (fits NP750XQA) [encompass.com] - single/summary-level source; verify.</t>
         </is>
       </c>
     </row>
@@ -3468,79 +3492,83 @@
       </c>
     </row>
     <row r="119">
-      <c r="A119" s="4" t="inlineStr">
-        <is>
-          <t>Samsung</t>
-        </is>
-      </c>
-      <c r="B119" s="4" t="inlineStr">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>Samsung</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
         <is>
           <t>BN39-02207G</t>
         </is>
       </c>
-      <c r="C119" s="4" t="inlineStr">
+      <c r="C119" t="inlineStr">
         <is>
           <t>Samsung TV Power Lead Connector - BN39-02207G</t>
         </is>
       </c>
-      <c r="D119" s="4" t="inlineStr">
-        <is>
-          <t>Medium (revision of confirmed part)</t>
-        </is>
-      </c>
-      <c r="E119" s="4" t="inlineStr">
-        <is>
-          <t>Same base number as confirmed BN39-02207C (different suffix letter = revision); type taken from that part. Exact-number listing not found.</t>
+      <c r="D119" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E119" t="inlineStr">
+        <is>
+          <t>Exact PN found via extended search: "Lead Connector Power" (fits 75KS8000) [spares2repair.co.uk]</t>
         </is>
       </c>
     </row>
     <row r="120">
-      <c r="A120" s="3" t="inlineStr">
-        <is>
-          <t>Samsung</t>
-        </is>
-      </c>
-      <c r="B120" s="3" t="inlineStr">
+      <c r="A120" s="4" t="inlineStr">
+        <is>
+          <t>Samsung</t>
+        </is>
+      </c>
+      <c r="B120" s="4" t="inlineStr">
         <is>
           <t>AH81-15490A</t>
         </is>
       </c>
-      <c r="C120" s="3" t="n"/>
-      <c r="D120" s="3" t="inlineStr">
-        <is>
-          <t>Needs review</t>
-        </is>
-      </c>
-      <c r="E120" s="3" t="inlineStr">
-        <is>
-          <t>No listing and no reliable series pattern; not guessed.</t>
+      <c r="C120" s="4" t="inlineStr">
+        <is>
+          <t>Samsung Soundbar OLED Board Module Assembly - AH81-15490A</t>
+        </is>
+      </c>
+      <c r="D120" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E120" s="4" t="inlineStr">
+        <is>
+          <t>Exact PN found via extended search: "OLED board-module assembly (service part, as paraphrased in summary)" (fits HW-B53C/ZA) [partstore.encompass.com] - single/summary-level source; verify.</t>
         </is>
       </c>
     </row>
     <row r="121">
-      <c r="A121" s="2" t="inlineStr">
-        <is>
-          <t>Samsung</t>
-        </is>
-      </c>
-      <c r="B121" s="2" t="inlineStr">
+      <c r="A121" s="4" t="inlineStr">
+        <is>
+          <t>Samsung</t>
+        </is>
+      </c>
+      <c r="B121" s="4" t="inlineStr">
         <is>
           <t>BA98-03895A</t>
         </is>
       </c>
-      <c r="C121" s="2" t="inlineStr">
-        <is>
-          <t>Samsung Laptop Case Assembly - BA98-03895A</t>
-        </is>
-      </c>
-      <c r="D121" s="2" t="inlineStr">
-        <is>
-          <t>Low (inferred from series)</t>
-        </is>
-      </c>
-      <c r="E121" s="2" t="inlineStr">
-        <is>
-          <t>INFERRED: part type taken from the part-number series; this exact part was not found in any listing. Verify before publishing.</t>
+      <c r="C121" s="4" t="inlineStr">
+        <is>
+          <t>Samsung Laptop Rear Case Assembly - BA98-03895A</t>
+        </is>
+      </c>
+      <c r="D121" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E121" s="4" t="inlineStr">
+        <is>
+          <t>Exact PN found via extended search: "rear case assembly (as paraphrased in summary)" (fits NP935QNAKA2TT) [partsips.com] - single/summary-level source; verify.</t>
         </is>
       </c>
     </row>
@@ -3595,25 +3623,29 @@
       </c>
     </row>
     <row r="124">
-      <c r="A124" s="3" t="inlineStr">
-        <is>
-          <t>Samsung</t>
-        </is>
-      </c>
-      <c r="B124" s="3" t="inlineStr">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>Samsung</t>
+        </is>
+      </c>
+      <c r="B124" t="inlineStr">
         <is>
           <t>6031-001662</t>
         </is>
       </c>
-      <c r="C124" s="3" t="n"/>
-      <c r="D124" s="3" t="inlineStr">
-        <is>
-          <t>Needs review</t>
-        </is>
-      </c>
-      <c r="E124" s="3" t="inlineStr">
-        <is>
-          <t>No listing and no reliable series pattern; not guessed.</t>
+      <c r="C124" t="inlineStr">
+        <is>
+          <t>Samsung Washer Dryer Spring Washer - 6031-001662</t>
+        </is>
+      </c>
+      <c r="D124" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E124" t="inlineStr">
+        <is>
+          <t>Exact PN found via extended search: "WASHER-SPRING;SK5,NTR,T1,OD45,ID35.2,SPR" (fits WD18DB8995BZSA, WD90H19AHSSA, WF90F19ADSSA) [sydneyappliance.com.au]</t>
         </is>
       </c>
     </row>
@@ -3668,25 +3700,29 @@
       </c>
     </row>
     <row r="127">
-      <c r="A127" s="3" t="inlineStr">
-        <is>
-          <t>Samsung</t>
-        </is>
-      </c>
-      <c r="B127" s="3" t="inlineStr">
+      <c r="A127" s="4" t="inlineStr">
+        <is>
+          <t>Samsung</t>
+        </is>
+      </c>
+      <c r="B127" s="4" t="inlineStr">
         <is>
           <t>AH81-17927A</t>
         </is>
       </c>
-      <c r="C127" s="3" t="n"/>
-      <c r="D127" s="3" t="inlineStr">
-        <is>
-          <t>Needs review</t>
-        </is>
-      </c>
-      <c r="E127" s="3" t="inlineStr">
-        <is>
-          <t>No listing and no reliable series pattern; not guessed.</t>
+      <c r="C127" s="4" t="inlineStr">
+        <is>
+          <t>Samsung Soundbar Wall Mount Bracket - AH81-17927A</t>
+        </is>
+      </c>
+      <c r="D127" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E127" s="4" t="inlineStr">
+        <is>
+          <t>Exact PN found via extended search: "Bracket-Wall Mount" (fits HW-B750F) [bhphotovideo.com] - single/summary-level source; verify.</t>
         </is>
       </c>
     </row>
@@ -3714,29 +3750,29 @@
       </c>
     </row>
     <row r="129">
-      <c r="A129" s="4" t="inlineStr">
-        <is>
-          <t>Samsung</t>
-        </is>
-      </c>
-      <c r="B129" s="4" t="inlineStr">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>Samsung</t>
+        </is>
+      </c>
+      <c r="B129" t="inlineStr">
         <is>
           <t>BA98-03053D</t>
         </is>
       </c>
-      <c r="C129" s="4" t="inlineStr">
+      <c r="C129" t="inlineStr">
         <is>
           <t>Samsung Laptop Rear Rubber Foot Assembly - BA98-03053D</t>
         </is>
       </c>
-      <c r="D129" s="4" t="inlineStr">
-        <is>
-          <t>Medium (revision of confirmed part)</t>
-        </is>
-      </c>
-      <c r="E129" s="4" t="inlineStr">
-        <is>
-          <t>Same base number as confirmed BA98-03053A (different suffix letter = revision); type taken from that part. Exact-number listing not found.</t>
+      <c r="D129" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E129" t="inlineStr">
+        <is>
+          <t>Exact PN found via extended search: "ASSY RUBBER-FOOT_BACK;MARS2-13,SEC,SI,GR" (fits NP930QED Galaxy Book2 Pro 360) [eetgroup.com]</t>
         </is>
       </c>
     </row>
@@ -3872,75 +3908,83 @@
       </c>
     </row>
     <row r="135">
-      <c r="A135" s="3" t="inlineStr">
-        <is>
-          <t>Samsung</t>
-        </is>
-      </c>
-      <c r="B135" s="3" t="inlineStr">
+      <c r="A135" s="4" t="inlineStr">
+        <is>
+          <t>Samsung</t>
+        </is>
+      </c>
+      <c r="B135" s="4" t="inlineStr">
         <is>
           <t>AH81-15433A</t>
         </is>
       </c>
-      <c r="C135" s="3" t="n"/>
-      <c r="D135" s="3" t="inlineStr">
-        <is>
-          <t>Needs review</t>
-        </is>
-      </c>
-      <c r="E135" s="3" t="inlineStr">
-        <is>
-          <t>No listing and no reliable series pattern; not guessed.</t>
+      <c r="C135" s="4" t="inlineStr">
+        <is>
+          <t>Samsung Soundbar Woofer FFC Cable - AH81-15433A</t>
+        </is>
+      </c>
+      <c r="D135" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E135" s="4" t="inlineStr">
+        <is>
+          <t>Exact PN found via extended search: "FFC cable for the woofer (service part, as paraphrased in summary)" (fits HW-B53C/ZA, HW-B53M/ZA) [partstore.encompass.com] - single/summary-level source; verify.</t>
         </is>
       </c>
     </row>
     <row r="136">
-      <c r="A136" s="2" t="inlineStr">
-        <is>
-          <t>Samsung</t>
-        </is>
-      </c>
-      <c r="B136" s="2" t="inlineStr">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>Samsung</t>
+        </is>
+      </c>
+      <c r="B136" t="inlineStr">
         <is>
           <t>BN39-01650B</t>
         </is>
       </c>
-      <c r="C136" s="2" t="inlineStr">
-        <is>
-          <t>Samsung TV Cable - BN39-01650B</t>
-        </is>
-      </c>
-      <c r="D136" s="2" t="inlineStr">
-        <is>
-          <t>Low (inferred from series)</t>
-        </is>
-      </c>
-      <c r="E136" s="2" t="inlineStr">
-        <is>
-          <t>INFERRED: part type taken from the part-number series; this exact part was not found in any listing. Verify before publishing.</t>
+      <c r="C136" t="inlineStr">
+        <is>
+          <t>Samsung TV Sub Assembly Lead Connector - BN39-01650B</t>
+        </is>
+      </c>
+      <c r="D136" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E136" t="inlineStr">
+        <is>
+          <t>Exact PN found via extended search: "Lead Connector-Sub Assembly" [samsungpartsusa.com]</t>
         </is>
       </c>
     </row>
     <row r="137">
-      <c r="A137" s="3" t="inlineStr">
-        <is>
-          <t>Samsung</t>
-        </is>
-      </c>
-      <c r="B137" s="3" t="inlineStr">
+      <c r="A137" s="4" t="inlineStr">
+        <is>
+          <t>Samsung</t>
+        </is>
+      </c>
+      <c r="B137" s="4" t="inlineStr">
         <is>
           <t>BA83-06215A</t>
         </is>
       </c>
-      <c r="C137" s="3" t="n"/>
-      <c r="D137" s="3" t="inlineStr">
-        <is>
-          <t>Needs review</t>
-        </is>
-      </c>
-      <c r="E137" s="3" t="inlineStr">
-        <is>
-          <t>No listing and no reliable series pattern; not guessed.</t>
+      <c r="C137" s="4" t="inlineStr">
+        <is>
+          <t>Samsung Laptop Front Cover and Screen Assembly - BA83-06215A</t>
+        </is>
+      </c>
+      <c r="D137" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E137" s="4" t="inlineStr">
+        <is>
+          <t>Exact PN found via extended search: "laptop front cover and screen assembly (trade-data description, as paraphrased in summary)" [volza.com] - single/summary-level source; verify.</t>
         </is>
       </c>
     </row>
@@ -3991,52 +4035,56 @@
       </c>
     </row>
     <row r="140">
-      <c r="A140" s="3" t="inlineStr">
-        <is>
-          <t>Samsung</t>
-        </is>
-      </c>
-      <c r="B140" s="3" t="inlineStr">
+      <c r="A140" t="inlineStr">
+        <is>
+          <t>Samsung</t>
+        </is>
+      </c>
+      <c r="B140" t="inlineStr">
         <is>
           <t>AH81-13985A</t>
         </is>
       </c>
-      <c r="C140" s="3" t="n"/>
-      <c r="D140" s="3" t="inlineStr">
-        <is>
-          <t>Needs review</t>
-        </is>
-      </c>
-      <c r="E140" s="3" t="inlineStr">
-        <is>
-          <t>No listing and no reliable series pattern; not guessed.</t>
+      <c r="C140" t="inlineStr">
+        <is>
+          <t>Samsung Soundbar Subwoofer Assembly - AH81-13985A</t>
+        </is>
+      </c>
+      <c r="D140" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E140" t="inlineStr">
+        <is>
+          <t>Exact PN found via extended search: "Subwoofer Assy;Zz-Ps-Wr55" (fits HW-A550/ZA) [tvserviceparts.com]</t>
         </is>
       </c>
     </row>
     <row r="141">
-      <c r="A141" s="2" t="inlineStr">
-        <is>
-          <t>Samsung</t>
-        </is>
-      </c>
-      <c r="B141" s="2" t="inlineStr">
+      <c r="A141" s="4" t="inlineStr">
+        <is>
+          <t>Samsung</t>
+        </is>
+      </c>
+      <c r="B141" s="4" t="inlineStr">
         <is>
           <t>AH94-03727A</t>
         </is>
       </c>
-      <c r="C141" s="2" t="inlineStr">
-        <is>
-          <t>Samsung Soundbar PCB Assembly - AH94-03727A</t>
-        </is>
-      </c>
-      <c r="D141" s="2" t="inlineStr">
-        <is>
-          <t>Low (inferred from series)</t>
-        </is>
-      </c>
-      <c r="E141" s="2" t="inlineStr">
-        <is>
-          <t>INFERRED: part type taken from the part-number series; this exact part was not found in any listing. Verify before publishing.</t>
+      <c r="C141" s="4" t="inlineStr">
+        <is>
+          <t>Samsung Soundbar Main PCB Assembly - AH94-03727A</t>
+        </is>
+      </c>
+      <c r="D141" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E141" s="4" t="inlineStr">
+        <is>
+          <t>Exact PN found via extended search: "main circuit board assembly (as paraphrased in summary)" (fits HW-J7500R) [ued.net] - single/summary-level source; verify.</t>
         </is>
       </c>
     </row>
@@ -4068,29 +4116,29 @@
       </c>
     </row>
     <row r="143">
-      <c r="A143" s="2" t="inlineStr">
-        <is>
-          <t>Samsung</t>
-        </is>
-      </c>
-      <c r="B143" s="2" t="inlineStr">
+      <c r="A143" t="inlineStr">
+        <is>
+          <t>Samsung</t>
+        </is>
+      </c>
+      <c r="B143" t="inlineStr">
         <is>
           <t>6003-001908</t>
         </is>
       </c>
-      <c r="C143" s="2" t="inlineStr">
-        <is>
-          <t>Samsung Taptype Screw - 6003-001908</t>
-        </is>
-      </c>
-      <c r="D143" s="2" t="inlineStr">
-        <is>
-          <t>Low (inferred from series)</t>
-        </is>
-      </c>
-      <c r="E143" s="2" t="inlineStr">
-        <is>
-          <t>INFERRED: part type taken from the part-number series; this exact part was not found in any listing. Verify before publishing.</t>
+      <c r="C143" t="inlineStr">
+        <is>
+          <t>Samsung TV Screw - 6003-001908</t>
+        </is>
+      </c>
+      <c r="D143" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E143" t="inlineStr">
+        <is>
+          <t>Exact PN found via extended search: "šroub televize (TV screw)" [fixpart.cz]</t>
         </is>
       </c>
     </row>
@@ -4230,29 +4278,29 @@
       </c>
     </row>
     <row r="149">
-      <c r="A149" s="2" t="inlineStr">
-        <is>
-          <t>Samsung</t>
-        </is>
-      </c>
-      <c r="B149" s="2" t="inlineStr">
+      <c r="A149" s="4" t="inlineStr">
+        <is>
+          <t>Samsung</t>
+        </is>
+      </c>
+      <c r="B149" s="4" t="inlineStr">
         <is>
           <t>BA96-08690A</t>
         </is>
       </c>
-      <c r="C149" s="2" t="inlineStr">
-        <is>
-          <t>Samsung Laptop LCD Assembly - BA96-08690A</t>
-        </is>
-      </c>
-      <c r="D149" s="2" t="inlineStr">
-        <is>
-          <t>Low (inferred from series)</t>
-        </is>
-      </c>
-      <c r="E149" s="2" t="inlineStr">
-        <is>
-          <t>INFERRED: part type taken from the part-number series; this exact part was not found in any listing. Verify before publishing.</t>
+      <c r="C149" s="4" t="inlineStr">
+        <is>
+          <t>Samsung Laptop Battery - BA96-08690A</t>
+        </is>
+      </c>
+      <c r="D149" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E149" s="4" t="inlineStr">
+        <is>
+          <t>Exact PN found via extended search: "Battery (60W 3940mAh 17.88V)" (fits NP750XQA-KB2US) [compupartsolutions.com] - single/summary-level source; verify.</t>
         </is>
       </c>
     </row>
@@ -4353,48 +4401,56 @@
       </c>
     </row>
     <row r="154">
-      <c r="A154" s="3" t="inlineStr">
-        <is>
-          <t>Samsung</t>
-        </is>
-      </c>
-      <c r="B154" s="3" t="inlineStr">
+      <c r="A154" s="4" t="inlineStr">
+        <is>
+          <t>Samsung</t>
+        </is>
+      </c>
+      <c r="B154" s="4" t="inlineStr">
         <is>
           <t>AH82-02599A</t>
         </is>
       </c>
-      <c r="C154" s="3" t="n"/>
-      <c r="D154" s="3" t="inlineStr">
-        <is>
-          <t>Needs review</t>
-        </is>
-      </c>
-      <c r="E154" s="3" t="inlineStr">
-        <is>
-          <t>No listing and no reliable series pattern; not guessed.</t>
+      <c r="C154" s="4" t="inlineStr">
+        <is>
+          <t>Samsung Accessory Holder P Decoration - AH82-02599A</t>
+        </is>
+      </c>
+      <c r="D154" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E154" s="4" t="inlineStr">
+        <is>
+          <t>Exact PN found via extended search: "Accessory Holder P Decoration (A)" (fits Samsung HW-LS60D/ZA music frame soundbar) [impactcomputers.com] - single/summary-level source; verify.</t>
         </is>
       </c>
     </row>
     <row r="155">
-      <c r="A155" s="3" t="inlineStr">
-        <is>
-          <t>Samsung</t>
-        </is>
-      </c>
-      <c r="B155" s="3" t="inlineStr">
+      <c r="A155" s="4" t="inlineStr">
+        <is>
+          <t>Samsung</t>
+        </is>
+      </c>
+      <c r="B155" s="4" t="inlineStr">
         <is>
           <t>AH81-15208A</t>
         </is>
       </c>
-      <c r="C155" s="3" t="n"/>
-      <c r="D155" s="3" t="inlineStr">
-        <is>
-          <t>Needs review</t>
-        </is>
-      </c>
-      <c r="E155" s="3" t="inlineStr">
-        <is>
-          <t>No listing and no reliable series pattern; not guessed.</t>
+      <c r="C155" s="4" t="inlineStr">
+        <is>
+          <t>Samsung Switch Membrane Touch Film - AH81-15208A</t>
+        </is>
+      </c>
+      <c r="D155" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E155" s="4" t="inlineStr">
+        <is>
+          <t>Exact PN found via extended search: "Switch membrane touch film" (fits Samsung HW-S800B/ZA and HW-S800D/ZA soundbars) [impactcomputers.com] - single/summary-level source; verify.</t>
         </is>
       </c>
     </row>
@@ -4711,110 +4767,110 @@
       </c>
     </row>
     <row r="168">
-      <c r="A168" s="2" t="inlineStr">
-        <is>
-          <t>Samsung</t>
-        </is>
-      </c>
-      <c r="B168" s="2" t="inlineStr">
+      <c r="A168" t="inlineStr">
+        <is>
+          <t>Samsung</t>
+        </is>
+      </c>
+      <c r="B168" t="inlineStr">
         <is>
           <t>BN39-02096A</t>
         </is>
       </c>
-      <c r="C168" s="2" t="inlineStr">
-        <is>
-          <t>Samsung TV Cable - BN39-02096A</t>
-        </is>
-      </c>
-      <c r="D168" s="2" t="inlineStr">
-        <is>
-          <t>Low (inferred from series)</t>
-        </is>
-      </c>
-      <c r="E168" s="2" t="inlineStr">
-        <is>
-          <t>INFERRED: part type taken from the part-number series; this exact part was not found in any listing. Verify before publishing.</t>
+      <c r="C168" t="inlineStr">
+        <is>
+          <t>Samsung TV Backlight Lead Connector Cable - BN39-02096A</t>
+        </is>
+      </c>
+      <c r="D168" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E168" t="inlineStr">
+        <is>
+          <t>Exact PN found via extended search: "Cable-Lead Connector-Blu" (fits Samsung 48/49-inch models incl. UA48J5200AKXXS, UA49J5200AKXZN, UN48J5000AFXZA, UN49M530DAFXZA) [tvserviceparts.com]</t>
         </is>
       </c>
     </row>
     <row r="169">
-      <c r="A169" s="2" t="inlineStr">
-        <is>
-          <t>Samsung</t>
-        </is>
-      </c>
-      <c r="B169" s="2" t="inlineStr">
+      <c r="A169" s="4" t="inlineStr">
+        <is>
+          <t>Samsung</t>
+        </is>
+      </c>
+      <c r="B169" s="4" t="inlineStr">
         <is>
           <t>BN39-01787B</t>
         </is>
       </c>
-      <c r="C169" s="2" t="inlineStr">
-        <is>
-          <t>Samsung TV Cable - BN39-01787B</t>
-        </is>
-      </c>
-      <c r="D169" s="2" t="inlineStr">
-        <is>
-          <t>Low (inferred from series)</t>
-        </is>
-      </c>
-      <c r="E169" s="2" t="inlineStr">
-        <is>
-          <t>INFERRED: part type taken from the part-number series; this exact part was not found in any listing. Verify before publishing.</t>
+      <c r="C169" s="4" t="inlineStr">
+        <is>
+          <t>Samsung TV Lead Connector - BN39-01787B</t>
+        </is>
+      </c>
+      <c r="D169" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E169" s="4" t="inlineStr">
+        <is>
+          <t>Exact PN found via extended search: "Lead Connector" (fits Samsung UN55F8000BF/XZA (schematic location EC13)) [pcrichard.encompass.com] - single/summary-level source; verify.</t>
         </is>
       </c>
     </row>
     <row r="170">
-      <c r="A170" s="2" t="inlineStr">
-        <is>
-          <t>Samsung</t>
-        </is>
-      </c>
-      <c r="B170" s="2" t="inlineStr">
+      <c r="A170" s="4" t="inlineStr">
+        <is>
+          <t>Samsung</t>
+        </is>
+      </c>
+      <c r="B170" s="4" t="inlineStr">
         <is>
           <t>BN39-02400A</t>
         </is>
       </c>
-      <c r="C170" s="2" t="inlineStr">
-        <is>
-          <t>Samsung TV Cable - BN39-02400A</t>
-        </is>
-      </c>
-      <c r="D170" s="2" t="inlineStr">
-        <is>
-          <t>Low (inferred from series)</t>
-        </is>
-      </c>
-      <c r="E170" s="2" t="inlineStr">
-        <is>
-          <t>INFERRED: part type taken from the part-number series; this exact part was not found in any listing. Verify before publishing.</t>
+      <c r="C170" s="4" t="inlineStr">
+        <is>
+          <t>Samsung TV Dimming Lead Connector - BN39-02400A</t>
+        </is>
+      </c>
+      <c r="D170" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E170" s="4" t="inlineStr">
+        <is>
+          <t>Exact PN found via extended search: "Lead Connector-Dimming" [samsungpartsusa.com] - single/summary-level source; verify.</t>
         </is>
       </c>
     </row>
     <row r="171">
-      <c r="A171" s="2" t="inlineStr">
-        <is>
-          <t>Samsung</t>
-        </is>
-      </c>
-      <c r="B171" s="2" t="inlineStr">
+      <c r="A171" s="4" t="inlineStr">
+        <is>
+          <t>Samsung</t>
+        </is>
+      </c>
+      <c r="B171" s="4" t="inlineStr">
         <is>
           <t>BN39-02397A</t>
         </is>
       </c>
-      <c r="C171" s="2" t="inlineStr">
-        <is>
-          <t>Samsung TV Cable - BN39-02397A</t>
-        </is>
-      </c>
-      <c r="D171" s="2" t="inlineStr">
-        <is>
-          <t>Low (inferred from series)</t>
-        </is>
-      </c>
-      <c r="E171" s="2" t="inlineStr">
-        <is>
-          <t>INFERRED: part type taken from the part-number series; this exact part was not found in any listing. Verify before publishing.</t>
+      <c r="C171" s="4" t="inlineStr">
+        <is>
+          <t>Samsung TV Dimming Lead Connector - BN39-02397A</t>
+        </is>
+      </c>
+      <c r="D171" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E171" s="4" t="inlineStr">
+        <is>
+          <t>Exact PN found via extended search: "Lead Connector-Dimming" [samsungpartsusa.com] - single/summary-level source; verify.</t>
         </is>
       </c>
     </row>
@@ -4869,52 +4925,56 @@
       </c>
     </row>
     <row r="174">
-      <c r="A174" s="3" t="inlineStr">
-        <is>
-          <t>Samsung</t>
-        </is>
-      </c>
-      <c r="B174" s="3" t="inlineStr">
+      <c r="A174" s="4" t="inlineStr">
+        <is>
+          <t>Samsung</t>
+        </is>
+      </c>
+      <c r="B174" s="4" t="inlineStr">
         <is>
           <t>AH81-17928A</t>
         </is>
       </c>
-      <c r="C174" s="3" t="n"/>
-      <c r="D174" s="3" t="inlineStr">
-        <is>
-          <t>Needs review</t>
-        </is>
-      </c>
-      <c r="E174" s="3" t="inlineStr">
-        <is>
-          <t>No listing and no reliable series pattern; not guessed.</t>
+      <c r="C174" s="4" t="inlineStr">
+        <is>
+          <t>Samsung Soundbar Top Cover Assembly - AH81-17928A</t>
+        </is>
+      </c>
+      <c r="D174" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E174" s="4" t="inlineStr">
+        <is>
+          <t>Exact PN found via extended search: "Top cover assembly" (fits Samsung HW-Q60CF/ZA soundbar) [impactcomputers.com] - single/summary-level source; verify.</t>
         </is>
       </c>
     </row>
     <row r="175">
-      <c r="A175" s="2" t="inlineStr">
-        <is>
-          <t>Samsung</t>
-        </is>
-      </c>
-      <c r="B175" s="2" t="inlineStr">
+      <c r="A175" s="4" t="inlineStr">
+        <is>
+          <t>Samsung</t>
+        </is>
+      </c>
+      <c r="B175" s="4" t="inlineStr">
         <is>
           <t>AH91-09157B</t>
         </is>
       </c>
-      <c r="C175" s="2" t="inlineStr">
-        <is>
-          <t>Samsung Soundbar Speaker Assembly - AH91-09157B</t>
-        </is>
-      </c>
-      <c r="D175" s="2" t="inlineStr">
-        <is>
-          <t>Low (inferred from series)</t>
-        </is>
-      </c>
-      <c r="E175" s="2" t="inlineStr">
-        <is>
-          <t>INFERRED: part type taken from the part-number series; this exact part was not found in any listing. Verify before publishing.</t>
+      <c r="C175" s="4" t="inlineStr">
+        <is>
+          <t>Samsung Soundbar Subwoofer Speaker - AH91-09157B</t>
+        </is>
+      </c>
+      <c r="D175" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E175" s="4" t="inlineStr">
+        <is>
+          <t>Exact PN found via extended search: "Speaker Subwoofer (SBQ990C)" (fits Samsung HW-Q990C/ZA soundbar) [impactcomputers.com] - single/summary-level source; verify.</t>
         </is>
       </c>
     </row>
@@ -4946,25 +5006,29 @@
       </c>
     </row>
     <row r="177">
-      <c r="A177" s="3" t="inlineStr">
-        <is>
-          <t>Samsung</t>
-        </is>
-      </c>
-      <c r="B177" s="3" t="inlineStr">
+      <c r="A177" s="4" t="inlineStr">
+        <is>
+          <t>Samsung</t>
+        </is>
+      </c>
+      <c r="B177" s="4" t="inlineStr">
         <is>
           <t>AH85-01070A</t>
         </is>
       </c>
-      <c r="C177" s="3" t="n"/>
-      <c r="D177" s="3" t="inlineStr">
-        <is>
-          <t>Needs review</t>
-        </is>
-      </c>
-      <c r="E177" s="3" t="inlineStr">
-        <is>
-          <t>No listing and no reliable series pattern; not guessed.</t>
+      <c r="C177" s="4" t="inlineStr">
+        <is>
+          <t>Samsung Soundbar Wireless Module Transmitter - AH85-01070A</t>
+        </is>
+      </c>
+      <c r="D177" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E177" s="4" t="inlineStr">
+        <is>
+          <t>Exact PN found via extended search: "Wireless module transmitter" (fits Samsung HW-Q990F soundbar, WSA520S wireless module) [impactcomputers.com] - single/summary-level source; verify.</t>
         </is>
       </c>
     </row>
@@ -5015,25 +5079,29 @@
       </c>
     </row>
     <row r="180">
-      <c r="A180" s="3" t="inlineStr">
-        <is>
-          <t>Samsung</t>
-        </is>
-      </c>
-      <c r="B180" s="3" t="inlineStr">
+      <c r="A180" s="4" t="inlineStr">
+        <is>
+          <t>Samsung</t>
+        </is>
+      </c>
+      <c r="B180" s="4" t="inlineStr">
         <is>
           <t>AH82-02415A</t>
         </is>
       </c>
-      <c r="C180" s="3" t="n"/>
-      <c r="D180" s="3" t="inlineStr">
-        <is>
-          <t>Needs review</t>
-        </is>
-      </c>
-      <c r="E180" s="3" t="inlineStr">
-        <is>
-          <t>No listing and no reliable series pattern; not guessed.</t>
+      <c r="C180" s="4" t="inlineStr">
+        <is>
+          <t>Samsung Soundbar Bottom Cover Assembly - AH82-02415A</t>
+        </is>
+      </c>
+      <c r="D180" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E180" s="4" t="inlineStr">
+        <is>
+          <t>Exact PN found via extended search: "A/S ASSY-COVER P-BOTTOM ASSY,HW-Q990 (bottom cover assembly)" (fits Samsung HW-Q990 soundbar) [servicepacksamsung.com] - single/summary-level source; verify.</t>
         </is>
       </c>
     </row>
@@ -5230,25 +5298,29 @@
       </c>
     </row>
     <row r="189">
-      <c r="A189" s="3" t="inlineStr">
-        <is>
-          <t>Samsung</t>
-        </is>
-      </c>
-      <c r="B189" s="3" t="inlineStr">
+      <c r="A189" s="4" t="inlineStr">
+        <is>
+          <t>Samsung</t>
+        </is>
+      </c>
+      <c r="B189" s="4" t="inlineStr">
         <is>
           <t>AH81-15428A</t>
         </is>
       </c>
-      <c r="C189" s="3" t="n"/>
-      <c r="D189" s="3" t="inlineStr">
-        <is>
-          <t>Needs review</t>
-        </is>
-      </c>
-      <c r="E189" s="3" t="inlineStr">
-        <is>
-          <t>No listing and no reliable series pattern; not guessed.</t>
+      <c r="C189" s="4" t="inlineStr">
+        <is>
+          <t>Samsung Soundbar Main PCB - AH81-15428A</t>
+        </is>
+      </c>
+      <c r="D189" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E189" s="4" t="inlineStr">
+        <is>
+          <t>Exact PN found via extended search: "Main PCB (soundbar)" (fits Samsung HW-B550 / HW-B550/XY) [samsungparts.nz] - single/summary-level source; verify.</t>
         </is>
       </c>
     </row>
@@ -5403,29 +5475,29 @@
       </c>
     </row>
     <row r="196">
-      <c r="A196" s="2" t="inlineStr">
-        <is>
-          <t>Samsung</t>
-        </is>
-      </c>
-      <c r="B196" s="2" t="inlineStr">
+      <c r="A196" s="4" t="inlineStr">
+        <is>
+          <t>Samsung</t>
+        </is>
+      </c>
+      <c r="B196" s="4" t="inlineStr">
         <is>
           <t>AH94-03881K</t>
         </is>
       </c>
-      <c r="C196" s="2" t="inlineStr">
-        <is>
-          <t>Samsung Soundbar PCB Assembly - AH94-03881K</t>
-        </is>
-      </c>
-      <c r="D196" s="2" t="inlineStr">
-        <is>
-          <t>Low (inferred from series)</t>
-        </is>
-      </c>
-      <c r="E196" s="2" t="inlineStr">
-        <is>
-          <t>INFERRED: part type taken from the part-number series; this exact part was not found in any listing. Verify before publishing.</t>
+      <c r="C196" s="4" t="inlineStr">
+        <is>
+          <t>Samsung Soundbar Main PCB Assembly - AH94-03881K</t>
+        </is>
+      </c>
+      <c r="D196" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E196" s="4" t="inlineStr">
+        <is>
+          <t>Exact PN found via extended search: "ASSY PCB MAIN;SBQ950A" (fits SBQ950A soundbar) [ued.net] - single/summary-level source; verify.</t>
         </is>
       </c>
     </row>
@@ -5453,25 +5525,29 @@
       </c>
     </row>
     <row r="198">
-      <c r="A198" s="3" t="inlineStr">
-        <is>
-          <t>Samsung</t>
-        </is>
-      </c>
-      <c r="B198" s="3" t="inlineStr">
+      <c r="A198" s="4" t="inlineStr">
+        <is>
+          <t>Samsung</t>
+        </is>
+      </c>
+      <c r="B198" s="4" t="inlineStr">
         <is>
           <t>AH82-02430A</t>
         </is>
       </c>
-      <c r="C198" s="3" t="n"/>
-      <c r="D198" s="3" t="inlineStr">
-        <is>
-          <t>Needs review</t>
-        </is>
-      </c>
-      <c r="E198" s="3" t="inlineStr">
-        <is>
-          <t>No listing and no reliable series pattern; not guessed.</t>
+      <c r="C198" s="4" t="inlineStr">
+        <is>
+          <t>Samsung Soundbar Rear Left Speaker Assembly - AH82-02430A</t>
+        </is>
+      </c>
+      <c r="D198" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E198" s="4" t="inlineStr">
+        <is>
+          <t>Exact PN found via extended search: "Rear left speaker assembly" (fits Samsung HW-Q930C soundbar) [encompass.com] - single/summary-level source; verify.</t>
         </is>
       </c>
     </row>
@@ -5499,56 +5575,56 @@
       </c>
     </row>
     <row r="200">
-      <c r="A200" s="2" t="inlineStr">
-        <is>
-          <t>Samsung</t>
-        </is>
-      </c>
-      <c r="B200" s="2" t="inlineStr">
+      <c r="A200" s="4" t="inlineStr">
+        <is>
+          <t>Samsung</t>
+        </is>
+      </c>
+      <c r="B200" s="4" t="inlineStr">
         <is>
           <t>AH94-03898Y</t>
         </is>
       </c>
-      <c r="C200" s="2" t="inlineStr">
-        <is>
-          <t>Samsung Soundbar PCB Assembly - AH94-03898Y</t>
-        </is>
-      </c>
-      <c r="D200" s="2" t="inlineStr">
-        <is>
-          <t>Low (inferred from series)</t>
-        </is>
-      </c>
-      <c r="E200" s="2" t="inlineStr">
-        <is>
-          <t>INFERRED: part type taken from the part-number series; this exact part was not found in any listing. Verify before publishing.</t>
+      <c r="C200" s="4" t="inlineStr">
+        <is>
+          <t>Samsung Main PCB Assembly - AH94-03898Y</t>
+        </is>
+      </c>
+      <c r="D200" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E200" s="4" t="inlineStr">
+        <is>
+          <t>Exact PN found via extended search: "Assembly PCB Main" (fits unstated (sibling suffixes are SBQ930B soundbar boards; unconfirmed)) [samsungpartsgh.shop] - single/summary-level source; verify.</t>
         </is>
       </c>
     </row>
     <row r="201">
-      <c r="A201" s="2" t="inlineStr">
-        <is>
-          <t>Samsung</t>
-        </is>
-      </c>
-      <c r="B201" s="2" t="inlineStr">
+      <c r="A201" s="4" t="inlineStr">
+        <is>
+          <t>Samsung</t>
+        </is>
+      </c>
+      <c r="B201" s="4" t="inlineStr">
         <is>
           <t>AH94-03811G</t>
         </is>
       </c>
-      <c r="C201" s="2" t="inlineStr">
-        <is>
-          <t>Samsung Soundbar PCB Assembly - AH94-03811G</t>
-        </is>
-      </c>
-      <c r="D201" s="2" t="inlineStr">
-        <is>
-          <t>Low (inferred from series)</t>
-        </is>
-      </c>
-      <c r="E201" s="2" t="inlineStr">
-        <is>
-          <t>INFERRED: part type taken from the part-number series; this exact part was not found in any listing. Verify before publishing.</t>
+      <c r="C201" s="4" t="inlineStr">
+        <is>
+          <t>Samsung Soundbar Main PCB Assembly - AH94-03811G</t>
+        </is>
+      </c>
+      <c r="D201" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E201" s="4" t="inlineStr">
+        <is>
+          <t>Exact PN found via extended search: "ASSY PCB MAIN;HW-Q90R,ZA" (fits HW-Q90R (ZA)) [ued.net] - single/summary-level source; verify.</t>
         </is>
       </c>
     </row>
@@ -5580,29 +5656,29 @@
       </c>
     </row>
     <row r="203">
-      <c r="A203" s="2" t="inlineStr">
-        <is>
-          <t>Samsung</t>
-        </is>
-      </c>
-      <c r="B203" s="2" t="inlineStr">
+      <c r="A203" t="inlineStr">
+        <is>
+          <t>Samsung</t>
+        </is>
+      </c>
+      <c r="B203" t="inlineStr">
         <is>
           <t>AH59-02761A</t>
         </is>
       </c>
-      <c r="C203" s="2" t="inlineStr">
-        <is>
-          <t>Samsung AV Remote Control - AH59-02761A</t>
-        </is>
-      </c>
-      <c r="D203" s="2" t="inlineStr">
-        <is>
-          <t>Low (inferred from series)</t>
-        </is>
-      </c>
-      <c r="E203" s="2" t="inlineStr">
-        <is>
-          <t>INFERRED: part type taken from the part-number series; this exact part was not found in any listing. Verify before publishing.</t>
+      <c r="C203" t="inlineStr">
+        <is>
+          <t>Samsung Soundbar Tweeter Driver - AH59-02761A</t>
+        </is>
+      </c>
+      <c r="D203" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E203" t="inlineStr">
+        <is>
+          <t>Exact PN found via extended search: "Tweeter driver" (fits Samsung HW-MS650 / HW-N950 soundbar) [ebay.ca]</t>
         </is>
       </c>
     </row>
@@ -5657,52 +5733,56 @@
       </c>
     </row>
     <row r="206">
-      <c r="A206" s="2" t="inlineStr">
-        <is>
-          <t>Samsung</t>
-        </is>
-      </c>
-      <c r="B206" s="2" t="inlineStr">
+      <c r="A206" s="4" t="inlineStr">
+        <is>
+          <t>Samsung</t>
+        </is>
+      </c>
+      <c r="B206" s="4" t="inlineStr">
         <is>
           <t>BA97-12356A</t>
         </is>
       </c>
-      <c r="C206" s="2" t="inlineStr">
+      <c r="C206" s="4" t="inlineStr">
         <is>
           <t>Samsung Laptop Front Top Case Assembly - BA97-12356A</t>
         </is>
       </c>
-      <c r="D206" s="2" t="inlineStr">
-        <is>
-          <t>Low (inferred from series)</t>
-        </is>
-      </c>
-      <c r="E206" s="2" t="inlineStr">
-        <is>
-          <t>INFERRED: part type taken from the part-number series; this exact part was not found in any listing. Verify before publishing.</t>
+      <c r="D206" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E206" s="4" t="inlineStr">
+        <is>
+          <t>Exact PN found via extended search: "Assembly Case Front-Top_SVC;MARS2-15,SEC,RED" (fits Samsung NP950QEDKC2US laptop) [ued.net/samsungparts] - single/summary-level source; verify.</t>
         </is>
       </c>
     </row>
     <row r="207">
-      <c r="A207" s="3" t="inlineStr">
-        <is>
-          <t>Samsung</t>
-        </is>
-      </c>
-      <c r="B207" s="3" t="inlineStr">
+      <c r="A207" t="inlineStr">
+        <is>
+          <t>Samsung</t>
+        </is>
+      </c>
+      <c r="B207" t="inlineStr">
         <is>
           <t>402-000128</t>
         </is>
       </c>
-      <c r="C207" s="3" t="n"/>
-      <c r="D207" s="3" t="inlineStr">
-        <is>
-          <t>Needs review</t>
-        </is>
-      </c>
-      <c r="E207" s="3" t="inlineStr">
-        <is>
-          <t>No listing and no reliable series pattern; not guessed.</t>
+      <c r="C207" t="inlineStr">
+        <is>
+          <t>Samsung Rectifier Diode - 402-000128</t>
+        </is>
+      </c>
+      <c r="D207" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E207" t="inlineStr">
+        <is>
+          <t>Exact PN found via extended search: "DIODE-RECTIFIER" (fits unstated) [ebay.com]</t>
         </is>
       </c>
     </row>
@@ -5757,25 +5837,29 @@
       </c>
     </row>
     <row r="210">
-      <c r="A210" s="3" t="inlineStr">
-        <is>
-          <t>Samsung</t>
-        </is>
-      </c>
-      <c r="B210" s="3" t="inlineStr">
+      <c r="A210" s="4" t="inlineStr">
+        <is>
+          <t>Samsung</t>
+        </is>
+      </c>
+      <c r="B210" s="4" t="inlineStr">
         <is>
           <t>AH81-15426A</t>
         </is>
       </c>
-      <c r="C210" s="3" t="n"/>
-      <c r="D210" s="3" t="inlineStr">
-        <is>
-          <t>Needs review</t>
-        </is>
-      </c>
-      <c r="E210" s="3" t="inlineStr">
-        <is>
-          <t>No listing and no reliable series pattern; not guessed.</t>
+      <c r="C210" s="4" t="inlineStr">
+        <is>
+          <t>Samsung Soundbar Amp PCB Assembly - AH81-15426A</t>
+        </is>
+      </c>
+      <c r="D210" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E210" s="4" t="inlineStr">
+        <is>
+          <t>Exact PN found via extended search: "AMP PCB (service assembly)" (fits Samsung HW-Q65C/ZA soundbar) [partstore.encompass.com] - single/summary-level source; verify.</t>
         </is>
       </c>
     </row>
@@ -5888,25 +5972,29 @@
       </c>
     </row>
     <row r="215">
-      <c r="A215" s="3" t="inlineStr">
-        <is>
-          <t>Samsung</t>
-        </is>
-      </c>
-      <c r="B215" s="3" t="inlineStr">
+      <c r="A215" s="4" t="inlineStr">
+        <is>
+          <t>Samsung</t>
+        </is>
+      </c>
+      <c r="B215" s="4" t="inlineStr">
         <is>
           <t>6031-002163</t>
         </is>
       </c>
-      <c r="C215" s="3" t="n"/>
-      <c r="D215" s="3" t="inlineStr">
-        <is>
-          <t>Needs review</t>
-        </is>
-      </c>
-      <c r="E215" s="3" t="inlineStr">
-        <is>
-          <t>No listing and no reliable series pattern; not guessed.</t>
+      <c r="C215" s="4" t="inlineStr">
+        <is>
+          <t>Samsung Dishwasher Plain Washer - 6031-002163</t>
+        </is>
+      </c>
+      <c r="D215" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E215" s="4" t="inlineStr">
+        <is>
+          <t>Exact PN found via extended search: "WASHER-PLAIN;S45C,ID5.5,OD17,T1.0" (fits Samsung dishwasher DW80R9950QN/AA-00) [partsdr.com] - single/summary-level source; verify.</t>
         </is>
       </c>
     </row>
@@ -5984,29 +6072,29 @@
       </c>
     </row>
     <row r="219">
-      <c r="A219" s="2" t="inlineStr">
-        <is>
-          <t>Samsung</t>
-        </is>
-      </c>
-      <c r="B219" s="2" t="inlineStr">
+      <c r="A219" t="inlineStr">
+        <is>
+          <t>Samsung</t>
+        </is>
+      </c>
+      <c r="B219" t="inlineStr">
         <is>
           <t>3903-001339</t>
         </is>
       </c>
-      <c r="C219" s="2" t="inlineStr">
-        <is>
-          <t>Samsung Power Cord - 3903-001339</t>
-        </is>
-      </c>
-      <c r="D219" s="2" t="inlineStr">
-        <is>
-          <t>Low (inferred from series)</t>
-        </is>
-      </c>
-      <c r="E219" s="2" t="inlineStr">
-        <is>
-          <t>INFERRED: part type taken from the part-number series; this exact part was not found in any listing. Verify before publishing.</t>
+      <c r="C219" t="inlineStr">
+        <is>
+          <t>Samsung TV Power Cord - 3903-001339</t>
+        </is>
+      </c>
+      <c r="D219" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E219" t="inlineStr">
+        <is>
+          <t>Exact PN found via extended search: "TV power cord (Longwell LS-91, 10A 125V)" (fits Samsung QN85QN900FF / QN85QN900FFXZA) [paulstv.com]</t>
         </is>
       </c>
     </row>
@@ -6038,29 +6126,29 @@
       </c>
     </row>
     <row r="221">
-      <c r="A221" s="2" t="inlineStr">
-        <is>
-          <t>Samsung</t>
-        </is>
-      </c>
-      <c r="B221" s="2" t="inlineStr">
+      <c r="A221" t="inlineStr">
+        <is>
+          <t>Samsung</t>
+        </is>
+      </c>
+      <c r="B221" t="inlineStr">
         <is>
           <t>3903-001077</t>
         </is>
       </c>
-      <c r="C221" s="2" t="inlineStr">
-        <is>
-          <t>Samsung Power Cord - 3903-001077</t>
-        </is>
-      </c>
-      <c r="D221" s="2" t="inlineStr">
-        <is>
-          <t>Low (inferred from series)</t>
-        </is>
-      </c>
-      <c r="E221" s="2" t="inlineStr">
-        <is>
-          <t>INFERRED: part type taken from the part-number series; this exact part was not found in any listing. Verify before publishing.</t>
+      <c r="C221" t="inlineStr">
+        <is>
+          <t>Samsung TV Power Cord - 3903-001077</t>
+        </is>
+      </c>
+      <c r="D221" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E221" t="inlineStr">
+        <is>
+          <t>Exact PN found via extended search: "POWER CORD-DT" (fits unstated) [samsungpartsusa.com]</t>
         </is>
       </c>
     </row>
@@ -6169,56 +6257,56 @@
       </c>
     </row>
     <row r="226">
-      <c r="A226" s="2" t="inlineStr">
-        <is>
-          <t>Samsung</t>
-        </is>
-      </c>
-      <c r="B226" s="2" t="inlineStr">
+      <c r="A226" s="4" t="inlineStr">
+        <is>
+          <t>Samsung</t>
+        </is>
+      </c>
+      <c r="B226" s="4" t="inlineStr">
         <is>
           <t>BN39-02136A</t>
         </is>
       </c>
-      <c r="C226" s="2" t="inlineStr">
-        <is>
-          <t>Samsung TV Cable - BN39-02136A</t>
-        </is>
-      </c>
-      <c r="D226" s="2" t="inlineStr">
-        <is>
-          <t>Low (inferred from series)</t>
-        </is>
-      </c>
-      <c r="E226" s="2" t="inlineStr">
-        <is>
-          <t>INFERRED: part type taken from the part-number series; this exact part was not found in any listing. Verify before publishing.</t>
+      <c r="C226" s="4" t="inlineStr">
+        <is>
+          <t>Samsung TV Main Assembly Lead Connector - BN39-02136A</t>
+        </is>
+      </c>
+      <c r="D226" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E226" s="4" t="inlineStr">
+        <is>
+          <t>Exact PN found via extended search: "Lead connect (main assembly)" (fits Samsung UN50M5300AFXZA-DA01 TV) [searspartsdirect.com] - single/summary-level source; verify.</t>
         </is>
       </c>
     </row>
     <row r="227">
-      <c r="A227" s="2" t="inlineStr">
-        <is>
-          <t>Samsung</t>
-        </is>
-      </c>
-      <c r="B227" s="2" t="inlineStr">
+      <c r="A227" t="inlineStr">
+        <is>
+          <t>Samsung</t>
+        </is>
+      </c>
+      <c r="B227" t="inlineStr">
         <is>
           <t>3903-001124</t>
         </is>
       </c>
-      <c r="C227" s="2" t="inlineStr">
-        <is>
-          <t>Samsung Power Cord - 3903-001124</t>
-        </is>
-      </c>
-      <c r="D227" s="2" t="inlineStr">
-        <is>
-          <t>Low (inferred from series)</t>
-        </is>
-      </c>
-      <c r="E227" s="2" t="inlineStr">
-        <is>
-          <t>INFERRED: part type taken from the part-number series; this exact part was not found in any listing. Verify before publishing.</t>
+      <c r="C227" t="inlineStr">
+        <is>
+          <t>Samsung TV Power Cable - 3903-001124</t>
+        </is>
+      </c>
+      <c r="D227" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E227" t="inlineStr">
+        <is>
+          <t>Exact PN found via extended search: "Power cable for TV (black)" [samsung.com/br]</t>
         </is>
       </c>
     </row>
@@ -6235,7 +6323,7 @@
       </c>
       <c r="C228" s="4" t="inlineStr">
         <is>
-          <t>Samsung AC Adapter - AD44-00161A</t>
+          <t>Samsung Camcorder AC Adapter - AD44-00161A</t>
         </is>
       </c>
       <c r="D228" s="4" t="inlineStr">
@@ -6245,34 +6333,34 @@
       </c>
       <c r="E228" s="4" t="inlineStr">
         <is>
-          <t>samsungpartsusa.com page; part type from listing summary</t>
+          <t>Exact PN found via extended search: "AC adapter (camcorder, 5V 1.5A)" (fits Samsung HMX-H205/H220/H300, HMX-Q200 camcorders) [amazon.com] - single/summary-level source; verify.</t>
         </is>
       </c>
     </row>
     <row r="229">
-      <c r="A229" s="4" t="inlineStr">
-        <is>
-          <t>Samsung</t>
-        </is>
-      </c>
-      <c r="B229" s="4" t="inlineStr">
+      <c r="A229" t="inlineStr">
+        <is>
+          <t>Samsung</t>
+        </is>
+      </c>
+      <c r="B229" t="inlineStr">
         <is>
           <t>AH59-01138A</t>
         </is>
       </c>
-      <c r="C229" s="4" t="inlineStr">
-        <is>
-          <t>Samsung TV Remote Control (RM-HF920) - AH59-01138A</t>
-        </is>
-      </c>
-      <c r="D229" s="4" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="E229" s="4" t="inlineStr">
-        <is>
-          <t>samsungpartsusa.com page; part type from listing summary</t>
+      <c r="C229" t="inlineStr">
+        <is>
+          <t>Samsung TV Remote Control - AH59-01138A</t>
+        </is>
+      </c>
+      <c r="D229" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E229" t="inlineStr">
+        <is>
+          <t>Exact PN found via extended search: "Remote control RM-HF920" [samsungpartsusa.com]</t>
         </is>
       </c>
     </row>
@@ -6354,29 +6442,29 @@
       </c>
     </row>
     <row r="233">
-      <c r="A233" s="2" t="inlineStr">
-        <is>
-          <t>Samsung</t>
-        </is>
-      </c>
-      <c r="B233" s="2" t="inlineStr">
+      <c r="A233" s="4" t="inlineStr">
+        <is>
+          <t>Samsung</t>
+        </is>
+      </c>
+      <c r="B233" s="4" t="inlineStr">
         <is>
           <t>6003-001621</t>
         </is>
       </c>
-      <c r="C233" s="2" t="inlineStr">
-        <is>
-          <t>Samsung Taptype Screw - 6003-001621</t>
-        </is>
-      </c>
-      <c r="D233" s="2" t="inlineStr">
-        <is>
-          <t>Low (inferred from series)</t>
-        </is>
-      </c>
-      <c r="E233" s="2" t="inlineStr">
-        <is>
-          <t>INFERRED: part type taken from the part-number series; this exact part was not found in any listing. Verify before publishing.</t>
+      <c r="C233" s="4" t="inlineStr">
+        <is>
+          <t>Samsung TV Stand Taptype Screw - 6003-001621</t>
+        </is>
+      </c>
+      <c r="D233" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E233" s="4" t="inlineStr">
+        <is>
+          <t>Exact PN found via extended search: "Screw (tap type; TV stand screw)" (fits Samsung TVs (stand screws)) [amazon.com] - single/summary-level source; verify.</t>
         </is>
       </c>
     </row>
@@ -6431,98 +6519,110 @@
       </c>
     </row>
     <row r="236">
-      <c r="A236" s="4" t="inlineStr">
-        <is>
-          <t>Samsung</t>
-        </is>
-      </c>
-      <c r="B236" s="4" t="inlineStr">
+      <c r="A236" t="inlineStr">
+        <is>
+          <t>Samsung</t>
+        </is>
+      </c>
+      <c r="B236" t="inlineStr">
         <is>
           <t>3903-001129</t>
         </is>
       </c>
-      <c r="C236" s="4" t="inlineStr">
-        <is>
-          <t>Samsung Power Cord (DT) - 3903-001129</t>
-        </is>
-      </c>
-      <c r="D236" s="4" t="inlineStr">
+      <c r="C236" t="inlineStr">
+        <is>
+          <t>Samsung TV Power Cord - 3903-001129</t>
+        </is>
+      </c>
+      <c r="D236" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E236" t="inlineStr">
+        <is>
+          <t>Exact PN found via extended search: "Power cable/cord-DT television (GBR 2P-F 250V 2.5A, L30)" (fits Samsung TV) [fixpart.co.uk]</t>
+        </is>
+      </c>
+    </row>
+    <row r="237">
+      <c r="A237" t="inlineStr">
+        <is>
+          <t>Samsung</t>
+        </is>
+      </c>
+      <c r="B237" t="inlineStr">
+        <is>
+          <t>AH81-15132A</t>
+        </is>
+      </c>
+      <c r="C237" t="inlineStr">
+        <is>
+          <t>Samsung Soundbar FFC Cable - AH81-15132A</t>
+        </is>
+      </c>
+      <c r="D237" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E237" t="inlineStr">
+        <is>
+          <t>Exact PN found via extended search: "A/S-FFC cable" (fits Samsung HW-S800B soundbar) [encompass.com]</t>
+        </is>
+      </c>
+    </row>
+    <row r="238">
+      <c r="A238" s="4" t="inlineStr">
+        <is>
+          <t>Samsung</t>
+        </is>
+      </c>
+      <c r="B238" s="4" t="inlineStr">
+        <is>
+          <t>3001-002872</t>
+        </is>
+      </c>
+      <c r="C238" s="4" t="inlineStr">
+        <is>
+          <t>Samsung Refrigerator Speaker - 3001-002872</t>
+        </is>
+      </c>
+      <c r="D238" s="4" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="E236" s="4" t="inlineStr">
-        <is>
-          <t>samsungpartsusa.com page; part type from listing summary</t>
-        </is>
-      </c>
-    </row>
-    <row r="237">
-      <c r="A237" s="3" t="inlineStr">
-        <is>
-          <t>Samsung</t>
-        </is>
-      </c>
-      <c r="B237" s="3" t="inlineStr">
-        <is>
-          <t>AH81-15132A</t>
-        </is>
-      </c>
-      <c r="C237" s="3" t="n"/>
-      <c r="D237" s="3" t="inlineStr">
-        <is>
-          <t>Needs review</t>
-        </is>
-      </c>
-      <c r="E237" s="3" t="inlineStr">
-        <is>
-          <t>No listing and no reliable series pattern; not guessed.</t>
-        </is>
-      </c>
-    </row>
-    <row r="238">
-      <c r="A238" s="3" t="inlineStr">
-        <is>
-          <t>Samsung</t>
-        </is>
-      </c>
-      <c r="B238" s="3" t="inlineStr">
-        <is>
-          <t>3001-002872</t>
-        </is>
-      </c>
-      <c r="C238" s="3" t="n"/>
-      <c r="D238" s="3" t="inlineStr">
-        <is>
-          <t>Needs review</t>
-        </is>
-      </c>
-      <c r="E238" s="3" t="inlineStr">
-        <is>
-          <t>No listing and no reliable series pattern; not guessed.</t>
+      <c r="E238" s="4" t="inlineStr">
+        <is>
+          <t>Exact PN found via extended search: "Speaker (6 ohm 80dB)" (fits Samsung RF29DB9900QDAA refrigerator) [ereplacementparts.com] - single/summary-level source; verify.</t>
         </is>
       </c>
     </row>
     <row r="239">
-      <c r="A239" s="3" t="inlineStr">
-        <is>
-          <t>Samsung</t>
-        </is>
-      </c>
-      <c r="B239" s="3" t="inlineStr">
+      <c r="A239" s="4" t="inlineStr">
+        <is>
+          <t>Samsung</t>
+        </is>
+      </c>
+      <c r="B239" s="4" t="inlineStr">
         <is>
           <t>AH83-00486A</t>
         </is>
       </c>
-      <c r="C239" s="3" t="n"/>
-      <c r="D239" s="3" t="inlineStr">
-        <is>
-          <t>Needs review</t>
-        </is>
-      </c>
-      <c r="E239" s="3" t="inlineStr">
-        <is>
-          <t>No listing and no reliable series pattern; not guessed.</t>
+      <c r="C239" s="4" t="inlineStr">
+        <is>
+          <t>Samsung Speaker Wire - AH83-00486A</t>
+        </is>
+      </c>
+      <c r="D239" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E239" s="4" t="inlineStr">
+        <is>
+          <t>Exact PN found via extended search: "CKD-Speaker wire" [samsungersatzteile.com] - single/summary-level source; verify.</t>
         </is>
       </c>
     </row>
@@ -6554,48 +6654,56 @@
       </c>
     </row>
     <row r="241">
-      <c r="A241" s="3" t="inlineStr">
-        <is>
-          <t>Samsung</t>
-        </is>
-      </c>
-      <c r="B241" s="3" t="inlineStr">
+      <c r="A241" s="4" t="inlineStr">
+        <is>
+          <t>Samsung</t>
+        </is>
+      </c>
+      <c r="B241" s="4" t="inlineStr">
         <is>
           <t>AH64-05864A</t>
         </is>
       </c>
-      <c r="C241" s="3" t="n"/>
-      <c r="D241" s="3" t="inlineStr">
-        <is>
-          <t>Needs review</t>
-        </is>
-      </c>
-      <c r="E241" s="3" t="inlineStr">
-        <is>
-          <t>No listing and no reliable series pattern; not guessed.</t>
+      <c r="C241" s="4" t="inlineStr">
+        <is>
+          <t>Samsung Door Cover - AH64-05864A</t>
+        </is>
+      </c>
+      <c r="D241" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E241" s="4" t="inlineStr">
+        <is>
+          <t>Exact PN found via extended search: "Cover-door (ABS)" (fits Samsung MX-J630) [ued.net] - single/summary-level source; verify.</t>
         </is>
       </c>
     </row>
     <row r="242">
-      <c r="A242" s="3" t="inlineStr">
-        <is>
-          <t>Samsung</t>
-        </is>
-      </c>
-      <c r="B242" s="3" t="inlineStr">
+      <c r="A242" t="inlineStr">
+        <is>
+          <t>Samsung</t>
+        </is>
+      </c>
+      <c r="B242" t="inlineStr">
         <is>
           <t>AH81-17977A</t>
         </is>
       </c>
-      <c r="C242" s="3" t="n"/>
-      <c r="D242" s="3" t="inlineStr">
-        <is>
-          <t>Needs review</t>
-        </is>
-      </c>
-      <c r="E242" s="3" t="inlineStr">
-        <is>
-          <t>No listing and no reliable series pattern; not guessed.</t>
+      <c r="C242" t="inlineStr">
+        <is>
+          <t>Samsung Soundbar Subwoofer Woofer - AH81-17977A</t>
+        </is>
+      </c>
+      <c r="D242" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E242" t="inlineStr">
+        <is>
+          <t>Exact PN found via extended search: "Subwoofer woofer" (fits Samsung HW-Q60CF/ZA soundbar) [impactcomputers.com]</t>
         </is>
       </c>
     </row>
@@ -6627,25 +6735,29 @@
       </c>
     </row>
     <row r="244">
-      <c r="A244" s="3" t="inlineStr">
-        <is>
-          <t>Samsung</t>
-        </is>
-      </c>
-      <c r="B244" s="3" t="inlineStr">
+      <c r="A244" s="4" t="inlineStr">
+        <is>
+          <t>Samsung</t>
+        </is>
+      </c>
+      <c r="B244" s="4" t="inlineStr">
         <is>
           <t>2401-004663</t>
         </is>
       </c>
-      <c r="C244" s="3" t="n"/>
-      <c r="D244" s="3" t="inlineStr">
-        <is>
-          <t>Needs review</t>
-        </is>
-      </c>
-      <c r="E244" s="3" t="inlineStr">
-        <is>
-          <t>No listing and no reliable series pattern; not guessed.</t>
+      <c r="C244" s="4" t="inlineStr">
+        <is>
+          <t>Samsung Aluminum Capacitor - 2401-004663</t>
+        </is>
+      </c>
+      <c r="D244" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E244" s="4" t="inlineStr">
+        <is>
+          <t>Exact PN found via extended search: "C-AL (aluminum capacitor)" [ebay.com] - single/summary-level source; verify.</t>
         </is>
       </c>
     </row>
@@ -6704,56 +6816,56 @@
       </c>
     </row>
     <row r="247">
-      <c r="A247" s="2" t="inlineStr">
-        <is>
-          <t>Samsung</t>
-        </is>
-      </c>
-      <c r="B247" s="2" t="inlineStr">
+      <c r="A247" s="4" t="inlineStr">
+        <is>
+          <t>Samsung</t>
+        </is>
+      </c>
+      <c r="B247" s="4" t="inlineStr">
         <is>
           <t>6002-001160</t>
         </is>
       </c>
-      <c r="C247" s="2" t="inlineStr">
+      <c r="C247" s="4" t="inlineStr">
         <is>
           <t>Samsung Tapping Screw - 6002-001160</t>
         </is>
       </c>
-      <c r="D247" s="2" t="inlineStr">
-        <is>
-          <t>Low (inferred from series)</t>
-        </is>
-      </c>
-      <c r="E247" s="2" t="inlineStr">
-        <is>
-          <t>INFERRED: part type taken from the part-number series; this exact part was not found in any listing. Verify before publishing.</t>
+      <c r="D247" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E247" s="4" t="inlineStr">
+        <is>
+          <t>Exact PN found via extended search: "Screw-tapping TH,+,NO,2,M5,L16,PASS,STS4" (fits Samsung washers) [partsdr.com] - single/summary-level source; verify.</t>
         </is>
       </c>
     </row>
     <row r="248">
-      <c r="A248" s="2" t="inlineStr">
-        <is>
-          <t>Samsung</t>
-        </is>
-      </c>
-      <c r="B248" s="2" t="inlineStr">
+      <c r="A248" t="inlineStr">
+        <is>
+          <t>Samsung</t>
+        </is>
+      </c>
+      <c r="B248" t="inlineStr">
         <is>
           <t>3903-001173</t>
         </is>
       </c>
-      <c r="C248" s="2" t="inlineStr">
-        <is>
-          <t>Samsung Power Cord - 3903-001173</t>
-        </is>
-      </c>
-      <c r="D248" s="2" t="inlineStr">
-        <is>
-          <t>Low (inferred from series)</t>
-        </is>
-      </c>
-      <c r="E248" s="2" t="inlineStr">
-        <is>
-          <t>INFERRED: part type taken from the part-number series; this exact part was not found in any listing. Verify before publishing.</t>
+      <c r="C248" t="inlineStr">
+        <is>
+          <t>Samsung TV Power Cord Assembly - 3903-001173</t>
+        </is>
+      </c>
+      <c r="D248" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E248" t="inlineStr">
+        <is>
+          <t>Exact PN found via extended search: "Television CBF power cord assembly" [partsimple.com]</t>
         </is>
       </c>
     </row>
@@ -6785,29 +6897,29 @@
       </c>
     </row>
     <row r="250">
-      <c r="A250" s="2" t="inlineStr">
-        <is>
-          <t>Samsung</t>
-        </is>
-      </c>
-      <c r="B250" s="2" t="inlineStr">
+      <c r="A250" t="inlineStr">
+        <is>
+          <t>Samsung</t>
+        </is>
+      </c>
+      <c r="B250" t="inlineStr">
         <is>
           <t>3903-001296</t>
         </is>
       </c>
-      <c r="C250" s="2" t="inlineStr">
-        <is>
-          <t>Samsung Power Cord - 3903-001296</t>
-        </is>
-      </c>
-      <c r="D250" s="2" t="inlineStr">
-        <is>
-          <t>Low (inferred from series)</t>
-        </is>
-      </c>
-      <c r="E250" s="2" t="inlineStr">
-        <is>
-          <t>INFERRED: part type taken from the part-number series; this exact part was not found in any listing. Verify before publishing.</t>
+      <c r="C250" t="inlineStr">
+        <is>
+          <t>Samsung TV Power Cord - 3903-001296</t>
+        </is>
+      </c>
+      <c r="D250" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E250" t="inlineStr">
+        <is>
+          <t>Exact PN found via extended search: "Power cord DT (TV)" (fits select Samsung TVs) [samsungpartsusa.com]</t>
         </is>
       </c>
     </row>
@@ -6839,29 +6951,29 @@
       </c>
     </row>
     <row r="252">
-      <c r="A252" s="2" t="inlineStr">
-        <is>
-          <t>Samsung</t>
-        </is>
-      </c>
-      <c r="B252" s="2" t="inlineStr">
+      <c r="A252" s="4" t="inlineStr">
+        <is>
+          <t>Samsung</t>
+        </is>
+      </c>
+      <c r="B252" s="4" t="inlineStr">
         <is>
           <t>3903-001311</t>
         </is>
       </c>
-      <c r="C252" s="2" t="inlineStr">
-        <is>
-          <t>Samsung Power Cord - 3903-001311</t>
-        </is>
-      </c>
-      <c r="D252" s="2" t="inlineStr">
-        <is>
-          <t>Low (inferred from series)</t>
-        </is>
-      </c>
-      <c r="E252" s="2" t="inlineStr">
-        <is>
-          <t>INFERRED: part type taken from the part-number series; this exact part was not found in any listing. Verify before publishing.</t>
+      <c r="C252" s="4" t="inlineStr">
+        <is>
+          <t>Samsung TV Power Cord - 3903-001311</t>
+        </is>
+      </c>
+      <c r="D252" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E252" s="4" t="inlineStr">
+        <is>
+          <t>Exact PN found via extended search: "Power cord-DT" [ebay.com] - single/summary-level source; verify.</t>
         </is>
       </c>
     </row>
@@ -6970,25 +7082,29 @@
       </c>
     </row>
     <row r="257">
-      <c r="A257" s="3" t="inlineStr">
-        <is>
-          <t>Samsung</t>
-        </is>
-      </c>
-      <c r="B257" s="3" t="inlineStr">
+      <c r="A257" s="4" t="inlineStr">
+        <is>
+          <t>Samsung</t>
+        </is>
+      </c>
+      <c r="B257" s="4" t="inlineStr">
         <is>
           <t>1204-003747</t>
         </is>
       </c>
-      <c r="C257" s="3" t="n"/>
-      <c r="D257" s="3" t="inlineStr">
-        <is>
-          <t>Needs review</t>
-        </is>
-      </c>
-      <c r="E257" s="3" t="inlineStr">
-        <is>
-          <t>No listing and no reliable series pattern; not guessed.</t>
+      <c r="C257" s="4" t="inlineStr">
+        <is>
+          <t>Samsung TV Video Processor IC - 1204-003747</t>
+        </is>
+      </c>
+      <c r="D257" s="4" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E257" s="4" t="inlineStr">
+        <is>
+          <t>Exact PN found via extended search: "IC-Video process" [samsungpartsusa.com] - single/summary-level source; verify.</t>
         </is>
       </c>
     </row>

</xml_diff>